<commit_message>
Include the Not sure/N-A option in the questions Excel export
That option is injected by the assessment UI at render time rather than
stored in questions.js, so the export script needs to add it explicitly
as a 6th column to keep the workbook in sync with what respondents see.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/OMI_Questions_Review.xlsx
+++ b/OMI_Questions_Review.xlsx
@@ -430,7 +430,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J76"/>
+  <dimension ref="A1:K76"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -443,6 +443,7 @@
     <col width="34" customWidth="1" min="8" max="8"/>
     <col width="34" customWidth="1" min="9" max="9"/>
     <col width="34" customWidth="1" min="10" max="10"/>
+    <col width="34" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -496,6 +497,11 @@
           <t>Option 5 (score 5)</t>
         </is>
       </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>Option 6 (Not sure / N-A)</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -548,6 +554,11 @@
           <t>Full business transaction observability — IT metrics linked to business SLAs, failures trigger automated triage.</t>
         </is>
       </c>
+      <c r="K2" s="2" t="inlineStr">
+        <is>
+          <t>Not sure / not applicable to my role — I don’t have visibility into this</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -600,6 +611,11 @@
           <t>Under 5 minutes — ML-driven anomaly detection linked to business KPIs.</t>
         </is>
       </c>
+      <c r="K3" s="2" t="inlineStr">
+        <is>
+          <t>Not sure / not applicable to my role — I don’t have visibility into this</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -652,6 +668,11 @@
           <t>A unified Business Observability platform — IT and business share a single source of truth.</t>
         </is>
       </c>
+      <c r="K4" s="2" t="inlineStr">
+        <is>
+          <t>Not sure / not applicable to my role — I don’t have visibility into this</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -704,6 +725,11 @@
           <t>Fully automated synthetic testing in production and pre-prod with business-impact scoring per journey.</t>
         </is>
       </c>
+      <c r="K5" s="2" t="inlineStr">
+        <is>
+          <t>Not sure / not applicable to my role — I don’t have visibility into this</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -756,6 +782,11 @@
           <t>Full alignment — observability drives business SLA reporting, regulatory submissions, and P&amp;L impact assessments.</t>
         </is>
       </c>
+      <c r="K6" s="2" t="inlineStr">
+        <is>
+          <t>Not sure / not applicable to my role — I don’t have visibility into this</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -808,6 +839,11 @@
           <t>Full business transaction observability — IT metrics linked to business SLAs, failures trigger automated triage.</t>
         </is>
       </c>
+      <c r="K7" s="2" t="inlineStr">
+        <is>
+          <t>Not sure / not applicable to my role — I don’t have visibility into this</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -860,6 +896,11 @@
           <t>Under 5 minutes — ML-driven anomaly detection linked to business KPIs.</t>
         </is>
       </c>
+      <c r="K8" s="2" t="inlineStr">
+        <is>
+          <t>Not sure / not applicable to my role — I don’t have visibility into this</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -912,6 +953,11 @@
           <t>A unified Business Observability platform — IT and business share a single source of truth.</t>
         </is>
       </c>
+      <c r="K9" s="2" t="inlineStr">
+        <is>
+          <t>Not sure / not applicable to my role — I don’t have visibility into this</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -964,6 +1010,11 @@
           <t>Fully automated synthetic testing across all channels with business-impact scoring per journey.</t>
         </is>
       </c>
+      <c r="K10" s="2" t="inlineStr">
+        <is>
+          <t>Not sure / not applicable to my role — I don’t have visibility into this</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -1016,6 +1067,11 @@
           <t>Full alignment — observability drives regulatory submissions, SLA reporting, and business impact assessments.</t>
         </is>
       </c>
+      <c r="K11" s="2" t="inlineStr">
+        <is>
+          <t>Not sure / not applicable to my role — I don’t have visibility into this</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -1068,6 +1124,11 @@
           <t>Full business transaction observability — IT metrics linked to business SLAs, failures trigger automated triage.</t>
         </is>
       </c>
+      <c r="K12" s="2" t="inlineStr">
+        <is>
+          <t>Not sure / not applicable to my role — I don’t have visibility into this</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -1120,6 +1181,11 @@
           <t>Under 5 minutes — ML-driven anomaly detection linked to business KPIs.</t>
         </is>
       </c>
+      <c r="K13" s="2" t="inlineStr">
+        <is>
+          <t>Not sure / not applicable to my role — I don’t have visibility into this</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -1172,6 +1238,11 @@
           <t>A unified Business Observability platform — IT and business share a single source of truth.</t>
         </is>
       </c>
+      <c r="K14" s="2" t="inlineStr">
+        <is>
+          <t>Not sure / not applicable to my role — I don’t have visibility into this</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -1224,6 +1295,11 @@
           <t>Fully automated synthetic testing across all channels with business-impact scoring per journey.</t>
         </is>
       </c>
+      <c r="K15" s="2" t="inlineStr">
+        <is>
+          <t>Not sure / not applicable to my role — I don’t have visibility into this</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -1276,6 +1352,11 @@
           <t>Full alignment — observability directly feeds regulatory reporting, incident notifications, and board-level resilience scorecards.</t>
         </is>
       </c>
+      <c r="K16" s="2" t="inlineStr">
+        <is>
+          <t>Not sure / not applicable to my role — I don’t have visibility into this</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
@@ -1328,6 +1409,11 @@
           <t>Full payment orchestration observability — each instrument mapped to SLA targets, failures trigger automated triage.</t>
         </is>
       </c>
+      <c r="K17" s="2" t="inlineStr">
+        <is>
+          <t>Not sure / not applicable to my role — I don’t have visibility into this</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
@@ -1380,6 +1466,11 @@
           <t>Under 5 minutes — ML-driven anomaly detection linked to settlement SLAs.</t>
         </is>
       </c>
+      <c r="K18" s="2" t="inlineStr">
+        <is>
+          <t>Not sure / not applicable to my role — I don’t have visibility into this</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
@@ -1432,6 +1523,11 @@
           <t>A unified payments observability platform — IT, finance, and compliance share one view.</t>
         </is>
       </c>
+      <c r="K19" s="2" t="inlineStr">
+        <is>
+          <t>Not sure / not applicable to my role — I don’t have visibility into this</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
@@ -1484,6 +1580,11 @@
           <t>All third-party dependencies are part of end-to-end transaction observability with business-impact scoring.</t>
         </is>
       </c>
+      <c r="K20" s="2" t="inlineStr">
+        <is>
+          <t>Not sure / not applicable to my role — I don’t have visibility into this</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
@@ -1536,6 +1637,11 @@
           <t>Full alignment — observability directly feeds regulatory reporting, merchant SLAs, and chargeback analysis.</t>
         </is>
       </c>
+      <c r="K21" s="2" t="inlineStr">
+        <is>
+          <t>Not sure / not applicable to my role — I don’t have visibility into this</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
@@ -1588,6 +1694,11 @@
           <t>Full payment orchestration observability — every instrument mapped to SLA targets, failures trigger automated triage.</t>
         </is>
       </c>
+      <c r="K22" s="2" t="inlineStr">
+        <is>
+          <t>Not sure / not applicable to my role — I don’t have visibility into this</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
@@ -1640,6 +1751,11 @@
           <t>Under 5 minutes — ML-driven anomaly detection linked to settlement SLAs.</t>
         </is>
       </c>
+      <c r="K23" s="2" t="inlineStr">
+        <is>
+          <t>Not sure / not applicable to my role — I don’t have visibility into this</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
@@ -1692,6 +1808,11 @@
           <t>A unified payments observability platform — IT, finance, and compliance share one live view.</t>
         </is>
       </c>
+      <c r="K24" s="2" t="inlineStr">
+        <is>
+          <t>Not sure / not applicable to my role — I don’t have visibility into this</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
@@ -1744,6 +1865,11 @@
           <t>All third-party dependencies are part of end-to-end transaction observability with business-impact scoring.</t>
         </is>
       </c>
+      <c r="K25" s="2" t="inlineStr">
+        <is>
+          <t>Not sure / not applicable to my role — I don’t have visibility into this</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
@@ -1796,6 +1922,11 @@
           <t>Full alignment — observability directly feeds scheme reporting, merchant SLA dashboards, and chargeback analysis.</t>
         </is>
       </c>
+      <c r="K26" s="2" t="inlineStr">
+        <is>
+          <t>Not sure / not applicable to my role — I don’t have visibility into this</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
@@ -1848,6 +1979,11 @@
           <t>Full citizen service observability — IT metrics linked to programme SLAs and citizen experience outcomes.</t>
         </is>
       </c>
+      <c r="K27" s="2" t="inlineStr">
+        <is>
+          <t>Not sure / not applicable to my role — I don’t have visibility into this</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
@@ -1900,6 +2036,11 @@
           <t>Under 5 minutes — ML-driven anomaly detection with automated escalation to the programme team.</t>
         </is>
       </c>
+      <c r="K28" s="2" t="inlineStr">
+        <is>
+          <t>Not sure / not applicable to my role — I don’t have visibility into this</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
@@ -1952,6 +2093,11 @@
           <t>A unified digital service observability platform — IT and programme management share one view.</t>
         </is>
       </c>
+      <c r="K29" s="2" t="inlineStr">
+        <is>
+          <t>Not sure / not applicable to my role — I don’t have visibility into this</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
@@ -2004,6 +2150,11 @@
           <t>Fully automated synthetic testing with business-impact scoring per citizen service.</t>
         </is>
       </c>
+      <c r="K30" s="2" t="inlineStr">
+        <is>
+          <t>Not sure / not applicable to my role — I don’t have visibility into this</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
@@ -2056,6 +2207,11 @@
           <t>Full alignment — observability feeds programme KPI dashboards, ministerial reporting, and audit submissions.</t>
         </is>
       </c>
+      <c r="K31" s="2" t="inlineStr">
+        <is>
+          <t>Not sure / not applicable to my role — I don’t have visibility into this</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
@@ -2108,6 +2264,11 @@
           <t>Full citizen service observability — IT metrics linked to programme SLAs and citizen experience outcomes.</t>
         </is>
       </c>
+      <c r="K32" s="2" t="inlineStr">
+        <is>
+          <t>Not sure / not applicable to my role — I don’t have visibility into this</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
@@ -2160,6 +2321,11 @@
           <t>Under 5 minutes — ML-driven anomaly detection with automated escalation to the programme team.</t>
         </is>
       </c>
+      <c r="K33" s="2" t="inlineStr">
+        <is>
+          <t>Not sure / not applicable to my role — I don’t have visibility into this</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
@@ -2212,6 +2378,11 @@
           <t>A unified digital service observability platform — IT and programme management share one live view.</t>
         </is>
       </c>
+      <c r="K34" s="2" t="inlineStr">
+        <is>
+          <t>Not sure / not applicable to my role — I don’t have visibility into this</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
@@ -2264,6 +2435,11 @@
           <t>Fully automated synthetic testing with business-impact scoring per citizen service.</t>
         </is>
       </c>
+      <c r="K35" s="2" t="inlineStr">
+        <is>
+          <t>Not sure / not applicable to my role — I don’t have visibility into this</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
@@ -2316,6 +2492,11 @@
           <t>Full alignment — observability feeds programme dashboards, ministerial reporting, and audit submissions.</t>
         </is>
       </c>
+      <c r="K36" s="2" t="inlineStr">
+        <is>
+          <t>Not sure / not applicable to my role — I don’t have visibility into this</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
@@ -2368,6 +2549,11 @@
           <t>Full product observability — every customer journey mapped to SLA targets with automated triage on failure.</t>
         </is>
       </c>
+      <c r="K37" s="2" t="inlineStr">
+        <is>
+          <t>Not sure / not applicable to my role — I don’t have visibility into this</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
@@ -2420,6 +2606,11 @@
           <t>Under 5 minutes — ML-driven anomaly detection with deployment context and customer impact scoring.</t>
         </is>
       </c>
+      <c r="K38" s="2" t="inlineStr">
+        <is>
+          <t>Not sure / not applicable to my role — I don’t have visibility into this</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
@@ -2472,6 +2663,11 @@
           <t>A unified product observability platform shared by engineering, CS, and account management.</t>
         </is>
       </c>
+      <c r="K39" s="2" t="inlineStr">
+        <is>
+          <t>Not sure / not applicable to my role — I don’t have visibility into this</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
@@ -2524,6 +2720,11 @@
           <t>Continuous synthetic testing in production and staging with business-impact scoring per journey.</t>
         </is>
       </c>
+      <c r="K40" s="2" t="inlineStr">
+        <is>
+          <t>Not sure / not applicable to my role — I don’t have visibility into this</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
@@ -2576,6 +2777,11 @@
           <t>Full alignment — observability feeds customer SLA reporting, renewal risk dashboards, and executive scorecards.</t>
         </is>
       </c>
+      <c r="K41" s="2" t="inlineStr">
+        <is>
+          <t>Not sure / not applicable to my role — I don’t have visibility into this</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
@@ -2628,6 +2834,11 @@
           <t>Full omnichannel transaction observability — every customer journey mapped to conversion and revenue KPIs with automated triage.</t>
         </is>
       </c>
+      <c r="K42" s="2" t="inlineStr">
+        <is>
+          <t>Not sure / not applicable to my role — I don’t have visibility into this</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
@@ -2680,6 +2891,11 @@
           <t>Under 5 minutes — ML-driven anomaly detection linked to GMV and conversion metrics.</t>
         </is>
       </c>
+      <c r="K43" s="2" t="inlineStr">
+        <is>
+          <t>Not sure / not applicable to my role — I don’t have visibility into this</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
@@ -2732,6 +2948,11 @@
           <t>A unified commerce observability platform — IT, merchandising, and commercial share one live view.</t>
         </is>
       </c>
+      <c r="K44" s="2" t="inlineStr">
+        <is>
+          <t>Not sure / not applicable to my role — I don’t have visibility into this</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
@@ -2784,6 +3005,11 @@
           <t>Continuous synthetic testing with GMV-impact scoring per journey degradation.</t>
         </is>
       </c>
+      <c r="K45" s="2" t="inlineStr">
+        <is>
+          <t>Not sure / not applicable to my role — I don’t have visibility into this</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
@@ -2836,6 +3062,11 @@
           <t>Full alignment — observability directly drives incident prioritisation, sale-event capacity planning, and P&amp;L impact reporting.</t>
         </is>
       </c>
+      <c r="K46" s="2" t="inlineStr">
+        <is>
+          <t>Not sure / not applicable to my role — I don’t have visibility into this</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
@@ -2888,6 +3119,11 @@
           <t>Full omnichannel transaction observability — every customer journey mapped to conversion and revenue KPIs with automated triage.</t>
         </is>
       </c>
+      <c r="K47" s="2" t="inlineStr">
+        <is>
+          <t>Not sure / not applicable to my role — I don’t have visibility into this</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
@@ -2940,6 +3176,11 @@
           <t>Under 5 minutes — ML-driven anomaly detection linked to GMV and conversion metrics.</t>
         </is>
       </c>
+      <c r="K48" s="2" t="inlineStr">
+        <is>
+          <t>Not sure / not applicable to my role — I don’t have visibility into this</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
@@ -2992,6 +3233,11 @@
           <t>A unified commerce observability platform — IT, merchandising, and commercial share one live view.</t>
         </is>
       </c>
+      <c r="K49" s="2" t="inlineStr">
+        <is>
+          <t>Not sure / not applicable to my role — I don’t have visibility into this</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
@@ -3044,6 +3290,11 @@
           <t>Continuous synthetic testing with GMV-impact scoring per journey degradation.</t>
         </is>
       </c>
+      <c r="K50" s="2" t="inlineStr">
+        <is>
+          <t>Not sure / not applicable to my role — I don’t have visibility into this</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
@@ -3096,6 +3347,11 @@
           <t>Full alignment — observability directly drives incident prioritisation, peak-event capacity planning, and revenue impact reporting.</t>
         </is>
       </c>
+      <c r="K51" s="2" t="inlineStr">
+        <is>
+          <t>Not sure / not applicable to my role — I don’t have visibility into this</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
@@ -3148,6 +3404,11 @@
           <t>Full end-to-end service observability — network, IT, and BSS metrics linked to subscriber experience KPIs with automated triage.</t>
         </is>
       </c>
+      <c r="K52" s="2" t="inlineStr">
+        <is>
+          <t>Not sure / not applicable to my role — I don’t have visibility into this</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
@@ -3200,6 +3461,11 @@
           <t>Under 5 minutes — ML-driven anomaly detection linked to subscriber experience and ARPU impact.</t>
         </is>
       </c>
+      <c r="K53" s="2" t="inlineStr">
+        <is>
+          <t>Not sure / not applicable to my role — I don’t have visibility into this</t>
+        </is>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
@@ -3252,6 +3518,11 @@
           <t>A unified telecom service observability platform shared across NOC, commercial, CX, and regulatory functions.</t>
         </is>
       </c>
+      <c r="K54" s="2" t="inlineStr">
+        <is>
+          <t>Not sure / not applicable to my role — I don’t have visibility into this</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
@@ -3304,6 +3575,11 @@
           <t>Continuous synthetic service testing with subscriber experience scoring and automated incident creation.</t>
         </is>
       </c>
+      <c r="K55" s="2" t="inlineStr">
+        <is>
+          <t>Not sure / not applicable to my role — I don’t have visibility into this</t>
+        </is>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
@@ -3356,6 +3632,11 @@
           <t>Full alignment — observability feeds TRAI regulatory submissions, interconnect SLA reporting, and subscriber experience dashboards.</t>
         </is>
       </c>
+      <c r="K56" s="2" t="inlineStr">
+        <is>
+          <t>Not sure / not applicable to my role — I don’t have visibility into this</t>
+        </is>
+      </c>
     </row>
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
@@ -3408,6 +3689,11 @@
           <t>Full end-to-end service observability — network, IT, and BSS metrics linked to subscriber experience KPIs with automated triage.</t>
         </is>
       </c>
+      <c r="K57" s="2" t="inlineStr">
+        <is>
+          <t>Not sure / not applicable to my role — I don’t have visibility into this</t>
+        </is>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
@@ -3460,6 +3746,11 @@
           <t>Under 5 minutes — ML-driven anomaly detection linked to subscriber experience and ARPU impact.</t>
         </is>
       </c>
+      <c r="K58" s="2" t="inlineStr">
+        <is>
+          <t>Not sure / not applicable to my role — I don’t have visibility into this</t>
+        </is>
+      </c>
     </row>
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
@@ -3512,6 +3803,11 @@
           <t>A unified telecom service observability platform shared across NOC, commercial, CX, and regulatory functions.</t>
         </is>
       </c>
+      <c r="K59" s="2" t="inlineStr">
+        <is>
+          <t>Not sure / not applicable to my role — I don’t have visibility into this</t>
+        </is>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
@@ -3564,6 +3860,11 @@
           <t>Continuous synthetic service testing with subscriber experience scoring and automated incident creation.</t>
         </is>
       </c>
+      <c r="K60" s="2" t="inlineStr">
+        <is>
+          <t>Not sure / not applicable to my role — I don’t have visibility into this</t>
+        </is>
+      </c>
     </row>
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
@@ -3616,6 +3917,11 @@
           <t>Full alignment — observability feeds regulatory submissions, interconnect SLA reporting, and subscriber experience dashboards.</t>
         </is>
       </c>
+      <c r="K61" s="2" t="inlineStr">
+        <is>
+          <t>Not sure / not applicable to my role — I don’t have visibility into this</t>
+        </is>
+      </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
@@ -3668,6 +3974,11 @@
           <t>Full operational transaction observability — SCADA, OMS, billing, and metering linked to regulatory SLAs with automated triage.</t>
         </is>
       </c>
+      <c r="K62" s="2" t="inlineStr">
+        <is>
+          <t>Not sure / not applicable to my role — I don’t have visibility into this</t>
+        </is>
+      </c>
     </row>
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
@@ -3720,6 +4031,11 @@
           <t>Under 5 minutes — ML-driven anomaly detection linked to grid SLAs and regulatory reliability indices.</t>
         </is>
       </c>
+      <c r="K63" s="2" t="inlineStr">
+        <is>
+          <t>Not sure / not applicable to my role — I don’t have visibility into this</t>
+        </is>
+      </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
@@ -3772,6 +4088,11 @@
           <t>A unified utility operations platform — grid, commercial, and regulatory teams share one live view.</t>
         </is>
       </c>
+      <c r="K64" s="2" t="inlineStr">
+        <is>
+          <t>Not sure / not applicable to my role — I don’t have visibility into this</t>
+        </is>
+      </c>
     </row>
     <row r="65">
       <c r="A65" s="2" t="inlineStr">
@@ -3824,6 +4145,11 @@
           <t>Continuous end-to-end operational monitoring with regulatory reliability impact scoring.</t>
         </is>
       </c>
+      <c r="K65" s="2" t="inlineStr">
+        <is>
+          <t>Not sure / not applicable to my role — I don’t have visibility into this</t>
+        </is>
+      </c>
     </row>
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
@@ -3876,6 +4202,11 @@
           <t>Full alignment — observability directly feeds regulatory submissions, SAIDI/SAIFI reporting, and tariff proceedings.</t>
         </is>
       </c>
+      <c r="K66" s="2" t="inlineStr">
+        <is>
+          <t>Not sure / not applicable to my role — I don’t have visibility into this</t>
+        </is>
+      </c>
     </row>
     <row r="67">
       <c r="A67" s="2" t="inlineStr">
@@ -3928,6 +4259,11 @@
           <t>Full operational transaction observability — SCADA, OMS, billing, and metering linked to regulatory SLAs with automated triage.</t>
         </is>
       </c>
+      <c r="K67" s="2" t="inlineStr">
+        <is>
+          <t>Not sure / not applicable to my role — I don’t have visibility into this</t>
+        </is>
+      </c>
     </row>
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
@@ -3980,6 +4316,11 @@
           <t>Under 5 minutes — ML-driven anomaly detection linked to grid SLAs and regulatory reliability indices.</t>
         </is>
       </c>
+      <c r="K68" s="2" t="inlineStr">
+        <is>
+          <t>Not sure / not applicable to my role — I don’t have visibility into this</t>
+        </is>
+      </c>
     </row>
     <row r="69">
       <c r="A69" s="2" t="inlineStr">
@@ -4032,6 +4373,11 @@
           <t>A unified utility operations platform — grid, commercial, and regulatory teams share one live view.</t>
         </is>
       </c>
+      <c r="K69" s="2" t="inlineStr">
+        <is>
+          <t>Not sure / not applicable to my role — I don’t have visibility into this</t>
+        </is>
+      </c>
     </row>
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
@@ -4084,6 +4430,11 @@
           <t>Continuous end-to-end operational monitoring with regulatory reliability impact scoring.</t>
         </is>
       </c>
+      <c r="K70" s="2" t="inlineStr">
+        <is>
+          <t>Not sure / not applicable to my role — I don’t have visibility into this</t>
+        </is>
+      </c>
     </row>
     <row r="71">
       <c r="A71" s="2" t="inlineStr">
@@ -4136,6 +4487,11 @@
           <t>Full alignment — observability directly feeds regulatory submissions, reliability index reporting, and tariff proceedings.</t>
         </is>
       </c>
+      <c r="K71" s="2" t="inlineStr">
+        <is>
+          <t>Not sure / not applicable to my role — I don’t have visibility into this</t>
+        </is>
+      </c>
     </row>
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
@@ -4188,6 +4544,11 @@
           <t>Full manufacturing transaction observability — ERP, MES, SCADA, and QMS metrics linked to delivery and quality SLAs with automated triage.</t>
         </is>
       </c>
+      <c r="K72" s="2" t="inlineStr">
+        <is>
+          <t>Not sure / not applicable to my role — I don’t have visibility into this</t>
+        </is>
+      </c>
     </row>
     <row r="73">
       <c r="A73" s="2" t="inlineStr">
@@ -4240,6 +4601,11 @@
           <t>Under 5 minutes — ML-driven anomaly detection linked to OEE and delivery SLA impact.</t>
         </is>
       </c>
+      <c r="K73" s="2" t="inlineStr">
+        <is>
+          <t>Not sure / not applicable to my role — I don’t have visibility into this</t>
+        </is>
+      </c>
     </row>
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
@@ -4292,6 +4658,11 @@
           <t>A unified manufacturing intelligence platform — operations, supply chain, quality, and commercial share one live view.</t>
         </is>
       </c>
+      <c r="K74" s="2" t="inlineStr">
+        <is>
+          <t>Not sure / not applicable to my role — I don’t have visibility into this</t>
+        </is>
+      </c>
     </row>
     <row r="75">
       <c r="A75" s="2" t="inlineStr">
@@ -4344,6 +4715,11 @@
           <t>Continuous end-to-end operational health monitoring with OEE and delivery commitment impact scoring.</t>
         </is>
       </c>
+      <c r="K75" s="2" t="inlineStr">
+        <is>
+          <t>Not sure / not applicable to my role — I don’t have visibility into this</t>
+        </is>
+      </c>
     </row>
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
@@ -4394,6 +4770,11 @@
       <c r="J76" s="2" t="inlineStr">
         <is>
           <t>Full alignment — observability directly drives incident prioritisation, capacity planning, and customer delivery SLA reporting.</t>
+        </is>
+      </c>
+      <c r="K76" s="2" t="inlineStr">
+        <is>
+          <t>Not sure / not applicable to my role — I don’t have visibility into this</t>
         </is>
       </c>
     </row>
@@ -4408,7 +4789,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J76"/>
+  <dimension ref="A1:K76"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -4421,6 +4802,7 @@
     <col width="34" customWidth="1" min="8" max="8"/>
     <col width="34" customWidth="1" min="9" max="9"/>
     <col width="34" customWidth="1" min="10" max="10"/>
+    <col width="34" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -4474,6 +4856,11 @@
           <t>Option 5 (score 5)</t>
         </is>
       </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>Option 6 (Not sure / N-A)</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -4526,6 +4913,11 @@
           <t>Automated retention controls, immutable storage, and on-demand regulatory reporting.</t>
         </is>
       </c>
+      <c r="K2" s="2" t="inlineStr">
+        <is>
+          <t>Not sure / not applicable to my role — I don’t have visibility into this</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -4578,6 +4970,11 @@
           <t>All regulatory-relevant logs on certified immutable storage with cryptographic integrity checks.</t>
         </is>
       </c>
+      <c r="K3" s="2" t="inlineStr">
+        <is>
+          <t>Not sure / not applicable to my role — I don’t have visibility into this</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -4630,6 +5027,11 @@
           <t>Within hours — automated audit-pack generation with a full chain of custody.</t>
         </is>
       </c>
+      <c r="K4" s="2" t="inlineStr">
+        <is>
+          <t>Not sure / not applicable to my role — I don’t have visibility into this</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -4682,6 +5084,11 @@
           <t>Zero-trust log access with MFA, just-in-time provisioning, and real-time access alerts.</t>
         </is>
       </c>
+      <c r="K5" s="2" t="inlineStr">
+        <is>
+          <t>Not sure / not applicable to my role — I don’t have visibility into this</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -4734,6 +5141,11 @@
           <t>Zero data egress enforced technically — all logs ingested, processed, and stored within the organisation perimeter.</t>
         </is>
       </c>
+      <c r="K6" s="2" t="inlineStr">
+        <is>
+          <t>Not sure / not applicable to my role — I don’t have visibility into this</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -4786,6 +5198,11 @@
           <t>Automated retention controls, immutable storage, and on-demand CBUAE/SAMA regulatory reporting.</t>
         </is>
       </c>
+      <c r="K7" s="2" t="inlineStr">
+        <is>
+          <t>Not sure / not applicable to my role — I don’t have visibility into this</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -4838,6 +5255,11 @@
           <t>All regulatory-relevant logs on certified immutable storage with cryptographic integrity verification.</t>
         </is>
       </c>
+      <c r="K8" s="2" t="inlineStr">
+        <is>
+          <t>Not sure / not applicable to my role — I don’t have visibility into this</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -4890,6 +5312,11 @@
           <t>Within hours — automated audit-pack generation with full chain of custody.</t>
         </is>
       </c>
+      <c r="K9" s="2" t="inlineStr">
+        <is>
+          <t>Not sure / not applicable to my role — I don’t have visibility into this</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -4942,6 +5369,11 @@
           <t>Zero-trust log access with MFA, just-in-time provisioning, and real-time access alerts for sensitive data.</t>
         </is>
       </c>
+      <c r="K10" s="2" t="inlineStr">
+        <is>
+          <t>Not sure / not applicable to my role — I don’t have visibility into this</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -4994,6 +5426,11 @@
           <t>Zero data egress enforced technically — all logs ingested, processed, and stored within the country perimeter.</t>
         </is>
       </c>
+      <c r="K11" s="2" t="inlineStr">
+        <is>
+          <t>Not sure / not applicable to my role — I don’t have visibility into this</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -5046,6 +5483,11 @@
           <t>Automated retention controls, immutable storage, and on-demand regulatory evidence packaging.</t>
         </is>
       </c>
+      <c r="K12" s="2" t="inlineStr">
+        <is>
+          <t>Not sure / not applicable to my role — I don’t have visibility into this</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -5098,6 +5540,11 @@
           <t>All regulatory-relevant logs on certified immutable storage with cryptographic integrity checks.</t>
         </is>
       </c>
+      <c r="K13" s="2" t="inlineStr">
+        <is>
+          <t>Not sure / not applicable to my role — I don’t have visibility into this</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -5150,6 +5597,11 @@
           <t>Within hours — automated audit-pack generation with a full chain of custody.</t>
         </is>
       </c>
+      <c r="K14" s="2" t="inlineStr">
+        <is>
+          <t>Not sure / not applicable to my role — I don’t have visibility into this</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -5202,6 +5654,11 @@
           <t>Zero-trust log access with MFA, just-in-time provisioning, and real-time access alerts for sensitive data.</t>
         </is>
       </c>
+      <c r="K15" s="2" t="inlineStr">
+        <is>
+          <t>Not sure / not applicable to my role — I don’t have visibility into this</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -5254,6 +5711,11 @@
           <t>Zero data egress enforced technically — all logs ingested, processed, and stored within the licensed jurisdiction.</t>
         </is>
       </c>
+      <c r="K16" s="2" t="inlineStr">
+        <is>
+          <t>Not sure / not applicable to my role — I don’t have visibility into this</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
@@ -5306,6 +5768,11 @@
           <t>Automated retention controls, immutable storage, and on-demand regulatory and settlement audit packs.</t>
         </is>
       </c>
+      <c r="K17" s="2" t="inlineStr">
+        <is>
+          <t>Not sure / not applicable to my role — I don’t have visibility into this</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
@@ -5358,6 +5825,11 @@
           <t>All payment-relevant logs on certified immutable storage with cryptographic integrity verification.</t>
         </is>
       </c>
+      <c r="K18" s="2" t="inlineStr">
+        <is>
+          <t>Not sure / not applicable to my role — I don’t have visibility into this</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
@@ -5410,6 +5882,11 @@
           <t>Within hours — automated dispute and audit-pack generation with chain of custody.</t>
         </is>
       </c>
+      <c r="K19" s="2" t="inlineStr">
+        <is>
+          <t>Not sure / not applicable to my role — I don’t have visibility into this</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
@@ -5462,6 +5939,11 @@
           <t>Zero-trust access with MFA, just-in-time provisioning, and real-time access alerts for payment data.</t>
         </is>
       </c>
+      <c r="K20" s="2" t="inlineStr">
+        <is>
+          <t>Not sure / not applicable to my role — I don’t have visibility into this</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
@@ -5514,6 +5996,11 @@
           <t>Zero data egress enforced technically with continuous compliance monitoring and annual PCI-DSS certification.</t>
         </is>
       </c>
+      <c r="K21" s="2" t="inlineStr">
+        <is>
+          <t>Not sure / not applicable to my role — I don’t have visibility into this</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
@@ -5566,6 +6053,11 @@
           <t>Automated retention controls, immutable storage, and on-demand PCI/scheme audit packs.</t>
         </is>
       </c>
+      <c r="K22" s="2" t="inlineStr">
+        <is>
+          <t>Not sure / not applicable to my role — I don’t have visibility into this</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
@@ -5618,6 +6110,11 @@
           <t>All in-scope payment logs on certified immutable storage with cryptographic integrity verification.</t>
         </is>
       </c>
+      <c r="K23" s="2" t="inlineStr">
+        <is>
+          <t>Not sure / not applicable to my role — I don’t have visibility into this</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
@@ -5670,6 +6167,11 @@
           <t>Within hours — automated dispute and audit-pack generation with chain of custody.</t>
         </is>
       </c>
+      <c r="K24" s="2" t="inlineStr">
+        <is>
+          <t>Not sure / not applicable to my role — I don’t have visibility into this</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
@@ -5722,6 +6224,11 @@
           <t>Zero-trust access with MFA, just-in-time provisioning, and real-time alerts for cardholder data access.</t>
         </is>
       </c>
+      <c r="K25" s="2" t="inlineStr">
+        <is>
+          <t>Not sure / not applicable to my role — I don’t have visibility into this</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
@@ -5774,6 +6281,11 @@
           <t>Zero data egress enforced technically with continuous compliance monitoring and annual certification.</t>
         </is>
       </c>
+      <c r="K26" s="2" t="inlineStr">
+        <is>
+          <t>Not sure / not applicable to my role — I don’t have visibility into this</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
@@ -5826,6 +6338,11 @@
           <t>Automated retention controls, immutable storage, and on-demand audit pack generation for all statutory requirements.</t>
         </is>
       </c>
+      <c r="K27" s="2" t="inlineStr">
+        <is>
+          <t>Not sure / not applicable to my role — I don’t have visibility into this</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
@@ -5878,6 +6395,11 @@
           <t>All in-scope logs on certified immutable storage with cryptographic integrity checks and chain of custody.</t>
         </is>
       </c>
+      <c r="K28" s="2" t="inlineStr">
+        <is>
+          <t>Not sure / not applicable to my role — I don’t have visibility into this</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
@@ -5930,6 +6452,11 @@
           <t>Within hours — automated audit pack generation with full chain of custody for statutory submissions.</t>
         </is>
       </c>
+      <c r="K29" s="2" t="inlineStr">
+        <is>
+          <t>Not sure / not applicable to my role — I don’t have visibility into this</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
@@ -5982,6 +6509,11 @@
           <t>Zero-trust log access with MFA, just-in-time provisioning, and automated alerts for sensitive data access.</t>
         </is>
       </c>
+      <c r="K30" s="2" t="inlineStr">
+        <is>
+          <t>Not sure / not applicable to my role — I don’t have visibility into this</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
@@ -6034,6 +6566,11 @@
           <t>Zero data egress enforced technically — all logs ingested, processed, and stored within approved government infrastructure.</t>
         </is>
       </c>
+      <c r="K31" s="2" t="inlineStr">
+        <is>
+          <t>Not sure / not applicable to my role — I don’t have visibility into this</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
@@ -6086,6 +6623,11 @@
           <t>Automated retention controls, immutable storage, and on-demand audit pack generation for all statutory requirements.</t>
         </is>
       </c>
+      <c r="K32" s="2" t="inlineStr">
+        <is>
+          <t>Not sure / not applicable to my role — I don’t have visibility into this</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
@@ -6138,6 +6680,11 @@
           <t>All in-scope logs on certified immutable storage with cryptographic integrity checks and chain of custody.</t>
         </is>
       </c>
+      <c r="K33" s="2" t="inlineStr">
+        <is>
+          <t>Not sure / not applicable to my role — I don’t have visibility into this</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
@@ -6190,6 +6737,11 @@
           <t>Within hours — automated audit pack generation with full chain of custody for statutory submissions.</t>
         </is>
       </c>
+      <c r="K34" s="2" t="inlineStr">
+        <is>
+          <t>Not sure / not applicable to my role — I don’t have visibility into this</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
@@ -6242,6 +6794,11 @@
           <t>Zero-trust log access with MFA, just-in-time provisioning, and automated alerts for sensitive citizen data access.</t>
         </is>
       </c>
+      <c r="K35" s="2" t="inlineStr">
+        <is>
+          <t>Not sure / not applicable to my role — I don’t have visibility into this</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
@@ -6294,6 +6851,11 @@
           <t>Zero data egress enforced technically — all logs ingested, processed, and stored within approved sovereign infrastructure.</t>
         </is>
       </c>
+      <c r="K36" s="2" t="inlineStr">
+        <is>
+          <t>Not sure / not applicable to my role — I don’t have visibility into this</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
@@ -6346,6 +6908,11 @@
           <t>Automated retention controls, immutable storage, and on-demand audit evidence generation for all certification scopes.</t>
         </is>
       </c>
+      <c r="K37" s="2" t="inlineStr">
+        <is>
+          <t>Not sure / not applicable to my role — I don’t have visibility into this</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
@@ -6398,6 +6965,11 @@
           <t>All in-scope logs on certified immutable storage with cryptographic integrity verification.</t>
         </is>
       </c>
+      <c r="K38" s="2" t="inlineStr">
+        <is>
+          <t>Not sure / not applicable to my role — I don’t have visibility into this</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
@@ -6450,6 +7022,11 @@
           <t>Within hours — automated evidence package generation with full chain of custody.</t>
         </is>
       </c>
+      <c r="K39" s="2" t="inlineStr">
+        <is>
+          <t>Not sure / not applicable to my role — I don’t have visibility into this</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
@@ -6502,6 +7079,11 @@
           <t>Zero-trust log access with MFA, just-in-time provisioning, and automated alerts for sensitive data access.</t>
         </is>
       </c>
+      <c r="K40" s="2" t="inlineStr">
+        <is>
+          <t>Not sure / not applicable to my role — I don’t have visibility into this</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
@@ -6554,6 +7136,11 @@
           <t>Zero data egress enforced technically — all logs ingested, processed, and stored within contractually required boundaries.</t>
         </is>
       </c>
+      <c r="K41" s="2" t="inlineStr">
+        <is>
+          <t>Not sure / not applicable to my role — I don’t have visibility into this</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
@@ -6606,6 +7193,11 @@
           <t>Automated retention controls, immutable storage, and on-demand PCI-DSS and DPDP audit evidence.</t>
         </is>
       </c>
+      <c r="K42" s="2" t="inlineStr">
+        <is>
+          <t>Not sure / not applicable to my role — I don’t have visibility into this</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
@@ -6658,6 +7250,11 @@
           <t>All in-scope logs on certified immutable storage with cryptographic integrity verification.</t>
         </is>
       </c>
+      <c r="K43" s="2" t="inlineStr">
+        <is>
+          <t>Not sure / not applicable to my role — I don’t have visibility into this</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
@@ -6710,6 +7307,11 @@
           <t>Within hours — automated evidence package generation with full chain of custody.</t>
         </is>
       </c>
+      <c r="K44" s="2" t="inlineStr">
+        <is>
+          <t>Not sure / not applicable to my role — I don’t have visibility into this</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
@@ -6762,6 +7364,11 @@
           <t>Zero-trust log access with MFA, just-in-time provisioning, and automated alerts for customer data access.</t>
         </is>
       </c>
+      <c r="K45" s="2" t="inlineStr">
+        <is>
+          <t>Not sure / not applicable to my role — I don’t have visibility into this</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
@@ -6814,6 +7421,11 @@
           <t>Zero data egress enforced technically with continuous compliance monitoring and PCI-DSS certification.</t>
         </is>
       </c>
+      <c r="K46" s="2" t="inlineStr">
+        <is>
+          <t>Not sure / not applicable to my role — I don’t have visibility into this</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
@@ -6866,6 +7478,11 @@
           <t>Automated retention controls, immutable storage, and on-demand PCI-DSS and data protection audit evidence.</t>
         </is>
       </c>
+      <c r="K47" s="2" t="inlineStr">
+        <is>
+          <t>Not sure / not applicable to my role — I don’t have visibility into this</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
@@ -6918,6 +7535,11 @@
           <t>All in-scope logs on certified immutable storage with cryptographic integrity verification.</t>
         </is>
       </c>
+      <c r="K48" s="2" t="inlineStr">
+        <is>
+          <t>Not sure / not applicable to my role — I don’t have visibility into this</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
@@ -6970,6 +7592,11 @@
           <t>Within hours — automated evidence package generation with full chain of custody.</t>
         </is>
       </c>
+      <c r="K49" s="2" t="inlineStr">
+        <is>
+          <t>Not sure / not applicable to my role — I don’t have visibility into this</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
@@ -7022,6 +7649,11 @@
           <t>Zero-trust log access with MFA, just-in-time provisioning, and automated alerts for customer data access.</t>
         </is>
       </c>
+      <c r="K50" s="2" t="inlineStr">
+        <is>
+          <t>Not sure / not applicable to my role — I don’t have visibility into this</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
@@ -7074,6 +7706,11 @@
           <t>Zero data egress enforced technically with continuous compliance monitoring and PCI-DSS certification.</t>
         </is>
       </c>
+      <c r="K51" s="2" t="inlineStr">
+        <is>
+          <t>Not sure / not applicable to my role — I don’t have visibility into this</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
@@ -7126,6 +7763,11 @@
           <t>Automated retention controls, immutable storage, and on-demand DoT/TRAI/CERT-In audit packs.</t>
         </is>
       </c>
+      <c r="K52" s="2" t="inlineStr">
+        <is>
+          <t>Not sure / not applicable to my role — I don’t have visibility into this</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
@@ -7178,6 +7820,11 @@
           <t>All DoT-mandated records on certified immutable storage with cryptographic integrity and chain of custody.</t>
         </is>
       </c>
+      <c r="K53" s="2" t="inlineStr">
+        <is>
+          <t>Not sure / not applicable to my role — I don’t have visibility into this</t>
+        </is>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
@@ -7230,6 +7877,11 @@
           <t>Within hours — automated audit-pack and lawful interception evidence generation with full chain of custody.</t>
         </is>
       </c>
+      <c r="K54" s="2" t="inlineStr">
+        <is>
+          <t>Not sure / not applicable to my role — I don’t have visibility into this</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
@@ -7282,6 +7934,11 @@
           <t>Zero-trust access with MFA, just-in-time provisioning, and automated alerts for sensitive subscriber data access.</t>
         </is>
       </c>
+      <c r="K55" s="2" t="inlineStr">
+        <is>
+          <t>Not sure / not applicable to my role — I don’t have visibility into this</t>
+        </is>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
@@ -7334,6 +7991,11 @@
           <t>Zero data egress enforced technically — all subscriber data and CDRs ingested, processed, and stored within Indian jurisdiction.</t>
         </is>
       </c>
+      <c r="K56" s="2" t="inlineStr">
+        <is>
+          <t>Not sure / not applicable to my role — I don’t have visibility into this</t>
+        </is>
+      </c>
     </row>
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
@@ -7386,6 +8048,11 @@
           <t>Automated retention controls, immutable storage, and on-demand regulator and law enforcement audit packs.</t>
         </is>
       </c>
+      <c r="K57" s="2" t="inlineStr">
+        <is>
+          <t>Not sure / not applicable to my role — I don’t have visibility into this</t>
+        </is>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
@@ -7438,6 +8105,11 @@
           <t>All legally mandated records on certified immutable storage with cryptographic integrity and chain of custody.</t>
         </is>
       </c>
+      <c r="K58" s="2" t="inlineStr">
+        <is>
+          <t>Not sure / not applicable to my role — I don’t have visibility into this</t>
+        </is>
+      </c>
     </row>
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
@@ -7490,6 +8162,11 @@
           <t>Within hours — automated audit-pack and lawful interception evidence generation with full chain of custody.</t>
         </is>
       </c>
+      <c r="K59" s="2" t="inlineStr">
+        <is>
+          <t>Not sure / not applicable to my role — I don’t have visibility into this</t>
+        </is>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
@@ -7542,6 +8219,11 @@
           <t>Zero-trust access with MFA, just-in-time provisioning, and automated alerts for sensitive subscriber data access.</t>
         </is>
       </c>
+      <c r="K60" s="2" t="inlineStr">
+        <is>
+          <t>Not sure / not applicable to my role — I don’t have visibility into this</t>
+        </is>
+      </c>
     </row>
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
@@ -7594,6 +8276,11 @@
           <t>Zero data egress enforced technically — all subscriber data and CDRs stored within applicable jurisdictional boundaries.</t>
         </is>
       </c>
+      <c r="K61" s="2" t="inlineStr">
+        <is>
+          <t>Not sure / not applicable to my role — I don’t have visibility into this</t>
+        </is>
+      </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
@@ -7646,6 +8333,11 @@
           <t>Automated retention controls, immutable storage, and on-demand CERC/SERC/CERT-In audit packs.</t>
         </is>
       </c>
+      <c r="K62" s="2" t="inlineStr">
+        <is>
+          <t>Not sure / not applicable to my role — I don’t have visibility into this</t>
+        </is>
+      </c>
     </row>
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
@@ -7698,6 +8390,11 @@
           <t>All CII-relevant logs on certified immutable storage with cryptographic integrity checks and chain of custody.</t>
         </is>
       </c>
+      <c r="K63" s="2" t="inlineStr">
+        <is>
+          <t>Not sure / not applicable to my role — I don’t have visibility into this</t>
+        </is>
+      </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
@@ -7750,6 +8447,11 @@
           <t>Within hours — automated audit pack generation with full chain of custody for regulatory submissions.</t>
         </is>
       </c>
+      <c r="K64" s="2" t="inlineStr">
+        <is>
+          <t>Not sure / not applicable to my role — I don’t have visibility into this</t>
+        </is>
+      </c>
     </row>
     <row r="65">
       <c r="A65" s="2" t="inlineStr">
@@ -7802,6 +8504,11 @@
           <t>Zero-trust access across OT and IT with MFA, just-in-time provisioning, and automated alerts for sensitive access.</t>
         </is>
       </c>
+      <c r="K65" s="2" t="inlineStr">
+        <is>
+          <t>Not sure / not applicable to my role — I don’t have visibility into this</t>
+        </is>
+      </c>
     </row>
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
@@ -7854,6 +8561,11 @@
           <t>Zero data egress enforced technically — all operational and consumer data stored within Indian jurisdiction.</t>
         </is>
       </c>
+      <c r="K66" s="2" t="inlineStr">
+        <is>
+          <t>Not sure / not applicable to my role — I don’t have visibility into this</t>
+        </is>
+      </c>
     </row>
     <row r="67">
       <c r="A67" s="2" t="inlineStr">
@@ -7906,6 +8618,11 @@
           <t>Automated retention controls, immutable storage, and on-demand regulatory audit packs.</t>
         </is>
       </c>
+      <c r="K67" s="2" t="inlineStr">
+        <is>
+          <t>Not sure / not applicable to my role — I don’t have visibility into this</t>
+        </is>
+      </c>
     </row>
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
@@ -7958,6 +8675,11 @@
           <t>All in-scope logs on certified immutable storage with cryptographic integrity checks and chain of custody.</t>
         </is>
       </c>
+      <c r="K68" s="2" t="inlineStr">
+        <is>
+          <t>Not sure / not applicable to my role — I don’t have visibility into this</t>
+        </is>
+      </c>
     </row>
     <row r="69">
       <c r="A69" s="2" t="inlineStr">
@@ -8010,6 +8732,11 @@
           <t>Within hours — automated audit pack generation with full chain of custody for regulatory submissions.</t>
         </is>
       </c>
+      <c r="K69" s="2" t="inlineStr">
+        <is>
+          <t>Not sure / not applicable to my role — I don’t have visibility into this</t>
+        </is>
+      </c>
     </row>
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
@@ -8062,6 +8789,11 @@
           <t>Zero-trust access across OT and IT with MFA, just-in-time provisioning, and automated alerts for sensitive access.</t>
         </is>
       </c>
+      <c r="K70" s="2" t="inlineStr">
+        <is>
+          <t>Not sure / not applicable to my role — I don’t have visibility into this</t>
+        </is>
+      </c>
     </row>
     <row r="71">
       <c r="A71" s="2" t="inlineStr">
@@ -8114,6 +8846,11 @@
           <t>Zero data egress enforced technically — all operational and consumer data stored within applicable jurisdictional boundaries.</t>
         </is>
       </c>
+      <c r="K71" s="2" t="inlineStr">
+        <is>
+          <t>Not sure / not applicable to my role — I don’t have visibility into this</t>
+        </is>
+      </c>
     </row>
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
@@ -8166,6 +8903,11 @@
           <t>Automated retention controls, immutable storage, and on-demand evidence generation for all certification and regulatory scopes.</t>
         </is>
       </c>
+      <c r="K72" s="2" t="inlineStr">
+        <is>
+          <t>Not sure / not applicable to my role — I don’t have visibility into this</t>
+        </is>
+      </c>
     </row>
     <row r="73">
       <c r="A73" s="2" t="inlineStr">
@@ -8218,6 +8960,11 @@
           <t>All regulated production records on certified immutable storage with cryptographic integrity verification.</t>
         </is>
       </c>
+      <c r="K73" s="2" t="inlineStr">
+        <is>
+          <t>Not sure / not applicable to my role — I don’t have visibility into this</t>
+        </is>
+      </c>
     </row>
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
@@ -8270,6 +9017,11 @@
           <t>Within hours — automated evidence package generation with full production batch chain of custody.</t>
         </is>
       </c>
+      <c r="K74" s="2" t="inlineStr">
+        <is>
+          <t>Not sure / not applicable to my role — I don’t have visibility into this</t>
+        </is>
+      </c>
     </row>
     <row r="75">
       <c r="A75" s="2" t="inlineStr">
@@ -8322,6 +9074,11 @@
           <t>Zero-trust access with MFA, just-in-time provisioning, and automated alerts for sensitive production data access.</t>
         </is>
       </c>
+      <c r="K75" s="2" t="inlineStr">
+        <is>
+          <t>Not sure / not applicable to my role — I don’t have visibility into this</t>
+        </is>
+      </c>
     </row>
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
@@ -8372,6 +9129,11 @@
       <c r="J76" s="2" t="inlineStr">
         <is>
           <t>Full data lifecycle governance — production records, quality data, and supply chain data retained, protected, and accessible for audit, recall, and ESG reporting.</t>
+        </is>
+      </c>
+      <c r="K76" s="2" t="inlineStr">
+        <is>
+          <t>Not sure / not applicable to my role — I don’t have visibility into this</t>
         </is>
       </c>
     </row>
@@ -8386,7 +9148,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J16"/>
+  <dimension ref="A1:K16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -8399,6 +9161,7 @@
     <col width="34" customWidth="1" min="8" max="8"/>
     <col width="34" customWidth="1" min="9" max="9"/>
     <col width="34" customWidth="1" min="10" max="10"/>
+    <col width="34" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -8452,6 +9215,11 @@
           <t>Option 5 (score 5)</t>
         </is>
       </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>Option 6 (Not sure / N-A)</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -8504,6 +9272,11 @@
           <t>APM fully integrated with business observability; every service has SLOs tied to business SLAs.</t>
         </is>
       </c>
+      <c r="K2" s="2" t="inlineStr">
+        <is>
+          <t>Not sure / not applicable to my role — I don’t have visibility into this</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -8556,6 +9329,11 @@
           <t>Third-party dependencies are part of end-to-end observability with business-impact scoring.</t>
         </is>
       </c>
+      <c r="K3" s="2" t="inlineStr">
+        <is>
+          <t>Not sure / not applicable to my role — I don’t have visibility into this</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -8608,6 +9386,11 @@
           <t>Full tracing linked to business transaction outcomes and user session context.</t>
         </is>
       </c>
+      <c r="K4" s="2" t="inlineStr">
+        <is>
+          <t>Not sure / not applicable to my role — I don’t have visibility into this</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -8660,6 +9443,11 @@
           <t>SLOs are integrated with business impact — error-budget depletion triggers business escalation.</t>
         </is>
       </c>
+      <c r="K5" s="2" t="inlineStr">
+        <is>
+          <t>Not sure / not applicable to my role — I don’t have visibility into this</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -8712,6 +9500,11 @@
           <t>Full channel observability linked to transaction success rates and customer experience scores.</t>
         </is>
       </c>
+      <c r="K6" s="2" t="inlineStr">
+        <is>
+          <t>Not sure / not applicable to my role — I don’t have visibility into this</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -8764,6 +9557,11 @@
           <t>Fully automated infrastructure discovery with real-time topology maps and dependency graphs.</t>
         </is>
       </c>
+      <c r="K7" s="2" t="inlineStr">
+        <is>
+          <t>Not sure / not applicable to my role — I don’t have visibility into this</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -8816,6 +9614,11 @@
           <t>Full network observability integrated with transaction tracing — network issues linked to business impact.</t>
         </is>
       </c>
+      <c r="K8" s="2" t="inlineStr">
+        <is>
+          <t>Not sure / not applicable to my role — I don’t have visibility into this</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -8868,6 +9671,11 @@
           <t>ML-driven capacity intelligence linked to business growth forecasts.</t>
         </is>
       </c>
+      <c r="K9" s="2" t="inlineStr">
+        <is>
+          <t>Not sure / not applicable to my role — I don’t have visibility into this</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -8920,6 +9728,11 @@
           <t>Container, host, and network observability unified with workload context and auto-scaling telemetry.</t>
         </is>
       </c>
+      <c r="K10" s="2" t="inlineStr">
+        <is>
+          <t>Not sure / not applicable to my role — I don’t have visibility into this</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -8972,6 +9785,11 @@
           <t>Full DC-to-application observability with predictive alerts linked to risk posture.</t>
         </is>
       </c>
+      <c r="K11" s="2" t="inlineStr">
+        <is>
+          <t>Not sure / not applicable to my role — I don’t have visibility into this</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -9024,6 +9842,11 @@
           <t>Full log data lake — all systems, all tiers, with real-time streaming and fast query.</t>
         </is>
       </c>
+      <c r="K12" s="2" t="inlineStr">
+        <is>
+          <t>Not sure / not applicable to my role — I don’t have visibility into this</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -9076,6 +9899,11 @@
           <t>Tiered storage (hot/warm/cold) with regulatory-aligned retention and real-time query across all tiers.</t>
         </is>
       </c>
+      <c r="K13" s="2" t="inlineStr">
+        <is>
+          <t>Not sure / not applicable to my role — I don’t have visibility into this</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -9128,6 +9956,11 @@
           <t>ML anomaly detection, automated pattern clustering, and natural-language log query.</t>
         </is>
       </c>
+      <c r="K14" s="2" t="inlineStr">
+        <is>
+          <t>Not sure / not applicable to my role — I don’t have visibility into this</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -9180,6 +10013,11 @@
           <t>Fully managed log lifecycle with ML-driven tiering, deduplication, and per-source cost attribution.</t>
         </is>
       </c>
+      <c r="K15" s="2" t="inlineStr">
+        <is>
+          <t>Not sure / not applicable to my role — I don’t have visibility into this</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -9230,6 +10068,11 @@
       <c r="J16" s="2" t="inlineStr">
         <is>
           <t>ML-powered log intelligence — behavioural baselines, multi-source correlation, SOAR integration.</t>
+        </is>
+      </c>
+      <c r="K16" s="2" t="inlineStr">
+        <is>
+          <t>Not sure / not applicable to my role — I don’t have visibility into this</t>
         </is>
       </c>
     </row>
@@ -9244,7 +10087,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J166"/>
+  <dimension ref="A1:K166"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -9257,6 +10100,7 @@
     <col width="34" customWidth="1" min="8" max="8"/>
     <col width="34" customWidth="1" min="9" max="9"/>
     <col width="34" customWidth="1" min="10" max="10"/>
+    <col width="34" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -9310,6 +10154,11 @@
           <t>Option 5 (score 5)</t>
         </is>
       </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>Option 6 (Not sure / N-A)</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -9362,6 +10211,11 @@
           <t>Full business transaction observability — IT metrics linked to business SLAs, failures trigger automated triage.</t>
         </is>
       </c>
+      <c r="K2" s="2" t="inlineStr">
+        <is>
+          <t>Not sure / not applicable to my role — I don’t have visibility into this</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -9414,6 +10268,11 @@
           <t>Under 5 minutes — ML-driven anomaly detection linked to business KPIs.</t>
         </is>
       </c>
+      <c r="K3" s="2" t="inlineStr">
+        <is>
+          <t>Not sure / not applicable to my role — I don’t have visibility into this</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -9466,6 +10325,11 @@
           <t>A unified Business Observability platform — IT and business share a single source of truth.</t>
         </is>
       </c>
+      <c r="K4" s="2" t="inlineStr">
+        <is>
+          <t>Not sure / not applicable to my role — I don’t have visibility into this</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -9518,6 +10382,11 @@
           <t>Fully automated synthetic testing in production and pre-prod with business-impact scoring per journey.</t>
         </is>
       </c>
+      <c r="K5" s="2" t="inlineStr">
+        <is>
+          <t>Not sure / not applicable to my role — I don’t have visibility into this</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -9570,6 +10439,11 @@
           <t>Full alignment — observability drives business SLA reporting, regulatory submissions, and P&amp;L impact assessments.</t>
         </is>
       </c>
+      <c r="K6" s="2" t="inlineStr">
+        <is>
+          <t>Not sure / not applicable to my role — I don’t have visibility into this</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -9622,6 +10496,11 @@
           <t>Full business transaction observability — IT metrics linked to business SLAs, failures trigger automated triage.</t>
         </is>
       </c>
+      <c r="K7" s="2" t="inlineStr">
+        <is>
+          <t>Not sure / not applicable to my role — I don’t have visibility into this</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -9674,6 +10553,11 @@
           <t>Under 5 minutes — ML-driven anomaly detection linked to business KPIs.</t>
         </is>
       </c>
+      <c r="K8" s="2" t="inlineStr">
+        <is>
+          <t>Not sure / not applicable to my role — I don’t have visibility into this</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -9726,6 +10610,11 @@
           <t>A unified Business Observability platform — IT and business share a single source of truth.</t>
         </is>
       </c>
+      <c r="K9" s="2" t="inlineStr">
+        <is>
+          <t>Not sure / not applicable to my role — I don’t have visibility into this</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -9778,6 +10667,11 @@
           <t>Fully automated synthetic testing across all channels with business-impact scoring per journey.</t>
         </is>
       </c>
+      <c r="K10" s="2" t="inlineStr">
+        <is>
+          <t>Not sure / not applicable to my role — I don’t have visibility into this</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -9830,6 +10724,11 @@
           <t>Full alignment — observability drives regulatory submissions, SLA reporting, and business impact assessments.</t>
         </is>
       </c>
+      <c r="K11" s="2" t="inlineStr">
+        <is>
+          <t>Not sure / not applicable to my role — I don’t have visibility into this</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -9882,6 +10781,11 @@
           <t>Full business transaction observability — IT metrics linked to business SLAs, failures trigger automated triage.</t>
         </is>
       </c>
+      <c r="K12" s="2" t="inlineStr">
+        <is>
+          <t>Not sure / not applicable to my role — I don’t have visibility into this</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -9934,6 +10838,11 @@
           <t>Under 5 minutes — ML-driven anomaly detection linked to business KPIs.</t>
         </is>
       </c>
+      <c r="K13" s="2" t="inlineStr">
+        <is>
+          <t>Not sure / not applicable to my role — I don’t have visibility into this</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -9986,6 +10895,11 @@
           <t>A unified Business Observability platform — IT and business share a single source of truth.</t>
         </is>
       </c>
+      <c r="K14" s="2" t="inlineStr">
+        <is>
+          <t>Not sure / not applicable to my role — I don’t have visibility into this</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -10038,6 +10952,11 @@
           <t>Fully automated synthetic testing across all channels with business-impact scoring per journey.</t>
         </is>
       </c>
+      <c r="K15" s="2" t="inlineStr">
+        <is>
+          <t>Not sure / not applicable to my role — I don’t have visibility into this</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -10090,6 +11009,11 @@
           <t>Full alignment — observability directly feeds regulatory reporting, incident notifications, and board-level resilience scorecards.</t>
         </is>
       </c>
+      <c r="K16" s="2" t="inlineStr">
+        <is>
+          <t>Not sure / not applicable to my role — I don’t have visibility into this</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
@@ -10142,6 +11066,11 @@
           <t>Full payment orchestration observability — each instrument mapped to SLA targets, failures trigger automated triage.</t>
         </is>
       </c>
+      <c r="K17" s="2" t="inlineStr">
+        <is>
+          <t>Not sure / not applicable to my role — I don’t have visibility into this</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
@@ -10194,6 +11123,11 @@
           <t>Under 5 minutes — ML-driven anomaly detection linked to settlement SLAs.</t>
         </is>
       </c>
+      <c r="K18" s="2" t="inlineStr">
+        <is>
+          <t>Not sure / not applicable to my role — I don’t have visibility into this</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
@@ -10246,6 +11180,11 @@
           <t>A unified payments observability platform — IT, finance, and compliance share one view.</t>
         </is>
       </c>
+      <c r="K19" s="2" t="inlineStr">
+        <is>
+          <t>Not sure / not applicable to my role — I don’t have visibility into this</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
@@ -10298,6 +11237,11 @@
           <t>All third-party dependencies are part of end-to-end transaction observability with business-impact scoring.</t>
         </is>
       </c>
+      <c r="K20" s="2" t="inlineStr">
+        <is>
+          <t>Not sure / not applicable to my role — I don’t have visibility into this</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
@@ -10350,6 +11294,11 @@
           <t>Full alignment — observability directly feeds regulatory reporting, merchant SLAs, and chargeback analysis.</t>
         </is>
       </c>
+      <c r="K21" s="2" t="inlineStr">
+        <is>
+          <t>Not sure / not applicable to my role — I don’t have visibility into this</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
@@ -10402,6 +11351,11 @@
           <t>Full payment orchestration observability — every instrument mapped to SLA targets, failures trigger automated triage.</t>
         </is>
       </c>
+      <c r="K22" s="2" t="inlineStr">
+        <is>
+          <t>Not sure / not applicable to my role — I don’t have visibility into this</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
@@ -10454,6 +11408,11 @@
           <t>Under 5 minutes — ML-driven anomaly detection linked to settlement SLAs.</t>
         </is>
       </c>
+      <c r="K23" s="2" t="inlineStr">
+        <is>
+          <t>Not sure / not applicable to my role — I don’t have visibility into this</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
@@ -10506,6 +11465,11 @@
           <t>A unified payments observability platform — IT, finance, and compliance share one live view.</t>
         </is>
       </c>
+      <c r="K24" s="2" t="inlineStr">
+        <is>
+          <t>Not sure / not applicable to my role — I don’t have visibility into this</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
@@ -10558,6 +11522,11 @@
           <t>All third-party dependencies are part of end-to-end transaction observability with business-impact scoring.</t>
         </is>
       </c>
+      <c r="K25" s="2" t="inlineStr">
+        <is>
+          <t>Not sure / not applicable to my role — I don’t have visibility into this</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
@@ -10610,6 +11579,11 @@
           <t>Full alignment — observability directly feeds scheme reporting, merchant SLA dashboards, and chargeback analysis.</t>
         </is>
       </c>
+      <c r="K26" s="2" t="inlineStr">
+        <is>
+          <t>Not sure / not applicable to my role — I don’t have visibility into this</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
@@ -10662,6 +11636,11 @@
           <t>Full citizen service observability — IT metrics linked to programme SLAs and citizen experience outcomes.</t>
         </is>
       </c>
+      <c r="K27" s="2" t="inlineStr">
+        <is>
+          <t>Not sure / not applicable to my role — I don’t have visibility into this</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
@@ -10714,6 +11693,11 @@
           <t>Under 5 minutes — ML-driven anomaly detection with automated escalation to the programme team.</t>
         </is>
       </c>
+      <c r="K28" s="2" t="inlineStr">
+        <is>
+          <t>Not sure / not applicable to my role — I don’t have visibility into this</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
@@ -10766,6 +11750,11 @@
           <t>A unified digital service observability platform — IT and programme management share one view.</t>
         </is>
       </c>
+      <c r="K29" s="2" t="inlineStr">
+        <is>
+          <t>Not sure / not applicable to my role — I don’t have visibility into this</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
@@ -10818,6 +11807,11 @@
           <t>Fully automated synthetic testing with business-impact scoring per citizen service.</t>
         </is>
       </c>
+      <c r="K30" s="2" t="inlineStr">
+        <is>
+          <t>Not sure / not applicable to my role — I don’t have visibility into this</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
@@ -10870,6 +11864,11 @@
           <t>Full alignment — observability feeds programme KPI dashboards, ministerial reporting, and audit submissions.</t>
         </is>
       </c>
+      <c r="K31" s="2" t="inlineStr">
+        <is>
+          <t>Not sure / not applicable to my role — I don’t have visibility into this</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
@@ -10922,6 +11921,11 @@
           <t>Full citizen service observability — IT metrics linked to programme SLAs and citizen experience outcomes.</t>
         </is>
       </c>
+      <c r="K32" s="2" t="inlineStr">
+        <is>
+          <t>Not sure / not applicable to my role — I don’t have visibility into this</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
@@ -10974,6 +11978,11 @@
           <t>Under 5 minutes — ML-driven anomaly detection with automated escalation to the programme team.</t>
         </is>
       </c>
+      <c r="K33" s="2" t="inlineStr">
+        <is>
+          <t>Not sure / not applicable to my role — I don’t have visibility into this</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
@@ -11026,6 +12035,11 @@
           <t>A unified digital service observability platform — IT and programme management share one live view.</t>
         </is>
       </c>
+      <c r="K34" s="2" t="inlineStr">
+        <is>
+          <t>Not sure / not applicable to my role — I don’t have visibility into this</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
@@ -11078,6 +12092,11 @@
           <t>Fully automated synthetic testing with business-impact scoring per citizen service.</t>
         </is>
       </c>
+      <c r="K35" s="2" t="inlineStr">
+        <is>
+          <t>Not sure / not applicable to my role — I don’t have visibility into this</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
@@ -11130,6 +12149,11 @@
           <t>Full alignment — observability feeds programme dashboards, ministerial reporting, and audit submissions.</t>
         </is>
       </c>
+      <c r="K36" s="2" t="inlineStr">
+        <is>
+          <t>Not sure / not applicable to my role — I don’t have visibility into this</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
@@ -11182,6 +12206,11 @@
           <t>Full product observability — every customer journey mapped to SLA targets with automated triage on failure.</t>
         </is>
       </c>
+      <c r="K37" s="2" t="inlineStr">
+        <is>
+          <t>Not sure / not applicable to my role — I don’t have visibility into this</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
@@ -11234,6 +12263,11 @@
           <t>Under 5 minutes — ML-driven anomaly detection with deployment context and customer impact scoring.</t>
         </is>
       </c>
+      <c r="K38" s="2" t="inlineStr">
+        <is>
+          <t>Not sure / not applicable to my role — I don’t have visibility into this</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
@@ -11286,6 +12320,11 @@
           <t>A unified product observability platform shared by engineering, CS, and account management.</t>
         </is>
       </c>
+      <c r="K39" s="2" t="inlineStr">
+        <is>
+          <t>Not sure / not applicable to my role — I don’t have visibility into this</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
@@ -11338,6 +12377,11 @@
           <t>Continuous synthetic testing in production and staging with business-impact scoring per journey.</t>
         </is>
       </c>
+      <c r="K40" s="2" t="inlineStr">
+        <is>
+          <t>Not sure / not applicable to my role — I don’t have visibility into this</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
@@ -11390,6 +12434,11 @@
           <t>Full alignment — observability feeds customer SLA reporting, renewal risk dashboards, and executive scorecards.</t>
         </is>
       </c>
+      <c r="K41" s="2" t="inlineStr">
+        <is>
+          <t>Not sure / not applicable to my role — I don’t have visibility into this</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
@@ -11442,6 +12491,11 @@
           <t>Full omnichannel transaction observability — every customer journey mapped to conversion and revenue KPIs with automated triage.</t>
         </is>
       </c>
+      <c r="K42" s="2" t="inlineStr">
+        <is>
+          <t>Not sure / not applicable to my role — I don’t have visibility into this</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
@@ -11494,6 +12548,11 @@
           <t>Under 5 minutes — ML-driven anomaly detection linked to GMV and conversion metrics.</t>
         </is>
       </c>
+      <c r="K43" s="2" t="inlineStr">
+        <is>
+          <t>Not sure / not applicable to my role — I don’t have visibility into this</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
@@ -11546,6 +12605,11 @@
           <t>A unified commerce observability platform — IT, merchandising, and commercial share one live view.</t>
         </is>
       </c>
+      <c r="K44" s="2" t="inlineStr">
+        <is>
+          <t>Not sure / not applicable to my role — I don’t have visibility into this</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
@@ -11598,6 +12662,11 @@
           <t>Continuous synthetic testing with GMV-impact scoring per journey degradation.</t>
         </is>
       </c>
+      <c r="K45" s="2" t="inlineStr">
+        <is>
+          <t>Not sure / not applicable to my role — I don’t have visibility into this</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
@@ -11650,6 +12719,11 @@
           <t>Full alignment — observability directly drives incident prioritisation, sale-event capacity planning, and P&amp;L impact reporting.</t>
         </is>
       </c>
+      <c r="K46" s="2" t="inlineStr">
+        <is>
+          <t>Not sure / not applicable to my role — I don’t have visibility into this</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
@@ -11702,6 +12776,11 @@
           <t>Full omnichannel transaction observability — every customer journey mapped to conversion and revenue KPIs with automated triage.</t>
         </is>
       </c>
+      <c r="K47" s="2" t="inlineStr">
+        <is>
+          <t>Not sure / not applicable to my role — I don’t have visibility into this</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
@@ -11754,6 +12833,11 @@
           <t>Under 5 minutes — ML-driven anomaly detection linked to GMV and conversion metrics.</t>
         </is>
       </c>
+      <c r="K48" s="2" t="inlineStr">
+        <is>
+          <t>Not sure / not applicable to my role — I don’t have visibility into this</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
@@ -11806,6 +12890,11 @@
           <t>A unified commerce observability platform — IT, merchandising, and commercial share one live view.</t>
         </is>
       </c>
+      <c r="K49" s="2" t="inlineStr">
+        <is>
+          <t>Not sure / not applicable to my role — I don’t have visibility into this</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
@@ -11858,6 +12947,11 @@
           <t>Continuous synthetic testing with GMV-impact scoring per journey degradation.</t>
         </is>
       </c>
+      <c r="K50" s="2" t="inlineStr">
+        <is>
+          <t>Not sure / not applicable to my role — I don’t have visibility into this</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
@@ -11910,6 +13004,11 @@
           <t>Full alignment — observability directly drives incident prioritisation, peak-event capacity planning, and revenue impact reporting.</t>
         </is>
       </c>
+      <c r="K51" s="2" t="inlineStr">
+        <is>
+          <t>Not sure / not applicable to my role — I don’t have visibility into this</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
@@ -11962,6 +13061,11 @@
           <t>Full end-to-end service observability — network, IT, and BSS metrics linked to subscriber experience KPIs with automated triage.</t>
         </is>
       </c>
+      <c r="K52" s="2" t="inlineStr">
+        <is>
+          <t>Not sure / not applicable to my role — I don’t have visibility into this</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
@@ -12014,6 +13118,11 @@
           <t>Under 5 minutes — ML-driven anomaly detection linked to subscriber experience and ARPU impact.</t>
         </is>
       </c>
+      <c r="K53" s="2" t="inlineStr">
+        <is>
+          <t>Not sure / not applicable to my role — I don’t have visibility into this</t>
+        </is>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
@@ -12066,6 +13175,11 @@
           <t>A unified telecom service observability platform shared across NOC, commercial, CX, and regulatory functions.</t>
         </is>
       </c>
+      <c r="K54" s="2" t="inlineStr">
+        <is>
+          <t>Not sure / not applicable to my role — I don’t have visibility into this</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
@@ -12118,6 +13232,11 @@
           <t>Continuous synthetic service testing with subscriber experience scoring and automated incident creation.</t>
         </is>
       </c>
+      <c r="K55" s="2" t="inlineStr">
+        <is>
+          <t>Not sure / not applicable to my role — I don’t have visibility into this</t>
+        </is>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
@@ -12170,6 +13289,11 @@
           <t>Full alignment — observability feeds TRAI regulatory submissions, interconnect SLA reporting, and subscriber experience dashboards.</t>
         </is>
       </c>
+      <c r="K56" s="2" t="inlineStr">
+        <is>
+          <t>Not sure / not applicable to my role — I don’t have visibility into this</t>
+        </is>
+      </c>
     </row>
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
@@ -12222,6 +13346,11 @@
           <t>Full end-to-end service observability — network, IT, and BSS metrics linked to subscriber experience KPIs with automated triage.</t>
         </is>
       </c>
+      <c r="K57" s="2" t="inlineStr">
+        <is>
+          <t>Not sure / not applicable to my role — I don’t have visibility into this</t>
+        </is>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
@@ -12274,6 +13403,11 @@
           <t>Under 5 minutes — ML-driven anomaly detection linked to subscriber experience and ARPU impact.</t>
         </is>
       </c>
+      <c r="K58" s="2" t="inlineStr">
+        <is>
+          <t>Not sure / not applicable to my role — I don’t have visibility into this</t>
+        </is>
+      </c>
     </row>
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
@@ -12326,6 +13460,11 @@
           <t>A unified telecom service observability platform shared across NOC, commercial, CX, and regulatory functions.</t>
         </is>
       </c>
+      <c r="K59" s="2" t="inlineStr">
+        <is>
+          <t>Not sure / not applicable to my role — I don’t have visibility into this</t>
+        </is>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
@@ -12378,6 +13517,11 @@
           <t>Continuous synthetic service testing with subscriber experience scoring and automated incident creation.</t>
         </is>
       </c>
+      <c r="K60" s="2" t="inlineStr">
+        <is>
+          <t>Not sure / not applicable to my role — I don’t have visibility into this</t>
+        </is>
+      </c>
     </row>
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
@@ -12430,6 +13574,11 @@
           <t>Full alignment — observability feeds regulatory submissions, interconnect SLA reporting, and subscriber experience dashboards.</t>
         </is>
       </c>
+      <c r="K61" s="2" t="inlineStr">
+        <is>
+          <t>Not sure / not applicable to my role — I don’t have visibility into this</t>
+        </is>
+      </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
@@ -12482,6 +13631,11 @@
           <t>Full operational transaction observability — SCADA, OMS, billing, and metering linked to regulatory SLAs with automated triage.</t>
         </is>
       </c>
+      <c r="K62" s="2" t="inlineStr">
+        <is>
+          <t>Not sure / not applicable to my role — I don’t have visibility into this</t>
+        </is>
+      </c>
     </row>
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
@@ -12534,6 +13688,11 @@
           <t>Under 5 minutes — ML-driven anomaly detection linked to grid SLAs and regulatory reliability indices.</t>
         </is>
       </c>
+      <c r="K63" s="2" t="inlineStr">
+        <is>
+          <t>Not sure / not applicable to my role — I don’t have visibility into this</t>
+        </is>
+      </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
@@ -12586,6 +13745,11 @@
           <t>A unified utility operations platform — grid, commercial, and regulatory teams share one live view.</t>
         </is>
       </c>
+      <c r="K64" s="2" t="inlineStr">
+        <is>
+          <t>Not sure / not applicable to my role — I don’t have visibility into this</t>
+        </is>
+      </c>
     </row>
     <row r="65">
       <c r="A65" s="2" t="inlineStr">
@@ -12638,6 +13802,11 @@
           <t>Continuous end-to-end operational monitoring with regulatory reliability impact scoring.</t>
         </is>
       </c>
+      <c r="K65" s="2" t="inlineStr">
+        <is>
+          <t>Not sure / not applicable to my role — I don’t have visibility into this</t>
+        </is>
+      </c>
     </row>
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
@@ -12690,6 +13859,11 @@
           <t>Full alignment — observability directly feeds regulatory submissions, SAIDI/SAIFI reporting, and tariff proceedings.</t>
         </is>
       </c>
+      <c r="K66" s="2" t="inlineStr">
+        <is>
+          <t>Not sure / not applicable to my role — I don’t have visibility into this</t>
+        </is>
+      </c>
     </row>
     <row r="67">
       <c r="A67" s="2" t="inlineStr">
@@ -12742,6 +13916,11 @@
           <t>Full operational transaction observability — SCADA, OMS, billing, and metering linked to regulatory SLAs with automated triage.</t>
         </is>
       </c>
+      <c r="K67" s="2" t="inlineStr">
+        <is>
+          <t>Not sure / not applicable to my role — I don’t have visibility into this</t>
+        </is>
+      </c>
     </row>
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
@@ -12794,6 +13973,11 @@
           <t>Under 5 minutes — ML-driven anomaly detection linked to grid SLAs and regulatory reliability indices.</t>
         </is>
       </c>
+      <c r="K68" s="2" t="inlineStr">
+        <is>
+          <t>Not sure / not applicable to my role — I don’t have visibility into this</t>
+        </is>
+      </c>
     </row>
     <row r="69">
       <c r="A69" s="2" t="inlineStr">
@@ -12846,6 +14030,11 @@
           <t>A unified utility operations platform — grid, commercial, and regulatory teams share one live view.</t>
         </is>
       </c>
+      <c r="K69" s="2" t="inlineStr">
+        <is>
+          <t>Not sure / not applicable to my role — I don’t have visibility into this</t>
+        </is>
+      </c>
     </row>
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
@@ -12898,6 +14087,11 @@
           <t>Continuous end-to-end operational monitoring with regulatory reliability impact scoring.</t>
         </is>
       </c>
+      <c r="K70" s="2" t="inlineStr">
+        <is>
+          <t>Not sure / not applicable to my role — I don’t have visibility into this</t>
+        </is>
+      </c>
     </row>
     <row r="71">
       <c r="A71" s="2" t="inlineStr">
@@ -12950,6 +14144,11 @@
           <t>Full alignment — observability directly feeds regulatory submissions, reliability index reporting, and tariff proceedings.</t>
         </is>
       </c>
+      <c r="K71" s="2" t="inlineStr">
+        <is>
+          <t>Not sure / not applicable to my role — I don’t have visibility into this</t>
+        </is>
+      </c>
     </row>
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
@@ -13002,6 +14201,11 @@
           <t>Full manufacturing transaction observability — ERP, MES, SCADA, and QMS metrics linked to delivery and quality SLAs with automated triage.</t>
         </is>
       </c>
+      <c r="K72" s="2" t="inlineStr">
+        <is>
+          <t>Not sure / not applicable to my role — I don’t have visibility into this</t>
+        </is>
+      </c>
     </row>
     <row r="73">
       <c r="A73" s="2" t="inlineStr">
@@ -13054,6 +14258,11 @@
           <t>Under 5 minutes — ML-driven anomaly detection linked to OEE and delivery SLA impact.</t>
         </is>
       </c>
+      <c r="K73" s="2" t="inlineStr">
+        <is>
+          <t>Not sure / not applicable to my role — I don’t have visibility into this</t>
+        </is>
+      </c>
     </row>
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
@@ -13106,6 +14315,11 @@
           <t>A unified manufacturing intelligence platform — operations, supply chain, quality, and commercial share one live view.</t>
         </is>
       </c>
+      <c r="K74" s="2" t="inlineStr">
+        <is>
+          <t>Not sure / not applicable to my role — I don’t have visibility into this</t>
+        </is>
+      </c>
     </row>
     <row r="75">
       <c r="A75" s="2" t="inlineStr">
@@ -13158,6 +14372,11 @@
           <t>Continuous end-to-end operational health monitoring with OEE and delivery commitment impact scoring.</t>
         </is>
       </c>
+      <c r="K75" s="2" t="inlineStr">
+        <is>
+          <t>Not sure / not applicable to my role — I don’t have visibility into this</t>
+        </is>
+      </c>
     </row>
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
@@ -13210,6 +14429,11 @@
           <t>Full alignment — observability directly drives incident prioritisation, capacity planning, and customer delivery SLA reporting.</t>
         </is>
       </c>
+      <c r="K76" s="2" t="inlineStr">
+        <is>
+          <t>Not sure / not applicable to my role — I don’t have visibility into this</t>
+        </is>
+      </c>
     </row>
     <row r="77">
       <c r="A77" s="2" t="inlineStr">
@@ -13262,6 +14486,11 @@
           <t>APM fully integrated with business observability; every service has SLOs tied to business SLAs.</t>
         </is>
       </c>
+      <c r="K77" s="2" t="inlineStr">
+        <is>
+          <t>Not sure / not applicable to my role — I don’t have visibility into this</t>
+        </is>
+      </c>
     </row>
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
@@ -13314,6 +14543,11 @@
           <t>Third-party dependencies are part of end-to-end observability with business-impact scoring.</t>
         </is>
       </c>
+      <c r="K78" s="2" t="inlineStr">
+        <is>
+          <t>Not sure / not applicable to my role — I don’t have visibility into this</t>
+        </is>
+      </c>
     </row>
     <row r="79">
       <c r="A79" s="2" t="inlineStr">
@@ -13366,6 +14600,11 @@
           <t>Full tracing linked to business transaction outcomes and user session context.</t>
         </is>
       </c>
+      <c r="K79" s="2" t="inlineStr">
+        <is>
+          <t>Not sure / not applicable to my role — I don’t have visibility into this</t>
+        </is>
+      </c>
     </row>
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
@@ -13418,6 +14657,11 @@
           <t>SLOs are integrated with business impact — error-budget depletion triggers business escalation.</t>
         </is>
       </c>
+      <c r="K80" s="2" t="inlineStr">
+        <is>
+          <t>Not sure / not applicable to my role — I don’t have visibility into this</t>
+        </is>
+      </c>
     </row>
     <row r="81">
       <c r="A81" s="2" t="inlineStr">
@@ -13470,6 +14714,11 @@
           <t>Full channel observability linked to transaction success rates and customer experience scores.</t>
         </is>
       </c>
+      <c r="K81" s="2" t="inlineStr">
+        <is>
+          <t>Not sure / not applicable to my role — I don’t have visibility into this</t>
+        </is>
+      </c>
     </row>
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
@@ -13522,6 +14771,11 @@
           <t>Fully automated infrastructure discovery with real-time topology maps and dependency graphs.</t>
         </is>
       </c>
+      <c r="K82" s="2" t="inlineStr">
+        <is>
+          <t>Not sure / not applicable to my role — I don’t have visibility into this</t>
+        </is>
+      </c>
     </row>
     <row r="83">
       <c r="A83" s="2" t="inlineStr">
@@ -13574,6 +14828,11 @@
           <t>Full network observability integrated with transaction tracing — network issues linked to business impact.</t>
         </is>
       </c>
+      <c r="K83" s="2" t="inlineStr">
+        <is>
+          <t>Not sure / not applicable to my role — I don’t have visibility into this</t>
+        </is>
+      </c>
     </row>
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
@@ -13626,6 +14885,11 @@
           <t>ML-driven capacity intelligence linked to business growth forecasts.</t>
         </is>
       </c>
+      <c r="K84" s="2" t="inlineStr">
+        <is>
+          <t>Not sure / not applicable to my role — I don’t have visibility into this</t>
+        </is>
+      </c>
     </row>
     <row r="85">
       <c r="A85" s="2" t="inlineStr">
@@ -13678,6 +14942,11 @@
           <t>Container, host, and network observability unified with workload context and auto-scaling telemetry.</t>
         </is>
       </c>
+      <c r="K85" s="2" t="inlineStr">
+        <is>
+          <t>Not sure / not applicable to my role — I don’t have visibility into this</t>
+        </is>
+      </c>
     </row>
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
@@ -13730,6 +14999,11 @@
           <t>Full DC-to-application observability with predictive alerts linked to risk posture.</t>
         </is>
       </c>
+      <c r="K86" s="2" t="inlineStr">
+        <is>
+          <t>Not sure / not applicable to my role — I don’t have visibility into this</t>
+        </is>
+      </c>
     </row>
     <row r="87">
       <c r="A87" s="2" t="inlineStr">
@@ -13782,6 +15056,11 @@
           <t>Full log data lake — all systems, all tiers, with real-time streaming and fast query.</t>
         </is>
       </c>
+      <c r="K87" s="2" t="inlineStr">
+        <is>
+          <t>Not sure / not applicable to my role — I don’t have visibility into this</t>
+        </is>
+      </c>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
@@ -13834,6 +15113,11 @@
           <t>Tiered storage (hot/warm/cold) with regulatory-aligned retention and real-time query across all tiers.</t>
         </is>
       </c>
+      <c r="K88" s="2" t="inlineStr">
+        <is>
+          <t>Not sure / not applicable to my role — I don’t have visibility into this</t>
+        </is>
+      </c>
     </row>
     <row r="89">
       <c r="A89" s="2" t="inlineStr">
@@ -13886,6 +15170,11 @@
           <t>ML anomaly detection, automated pattern clustering, and natural-language log query.</t>
         </is>
       </c>
+      <c r="K89" s="2" t="inlineStr">
+        <is>
+          <t>Not sure / not applicable to my role — I don’t have visibility into this</t>
+        </is>
+      </c>
     </row>
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
@@ -13938,6 +15227,11 @@
           <t>Fully managed log lifecycle with ML-driven tiering, deduplication, and per-source cost attribution.</t>
         </is>
       </c>
+      <c r="K90" s="2" t="inlineStr">
+        <is>
+          <t>Not sure / not applicable to my role — I don’t have visibility into this</t>
+        </is>
+      </c>
     </row>
     <row r="91">
       <c r="A91" s="2" t="inlineStr">
@@ -13990,6 +15284,11 @@
           <t>ML-powered log intelligence — behavioural baselines, multi-source correlation, SOAR integration.</t>
         </is>
       </c>
+      <c r="K91" s="2" t="inlineStr">
+        <is>
+          <t>Not sure / not applicable to my role — I don’t have visibility into this</t>
+        </is>
+      </c>
     </row>
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
@@ -14042,6 +15341,11 @@
           <t>Automated retention controls, immutable storage, and on-demand regulatory reporting.</t>
         </is>
       </c>
+      <c r="K92" s="2" t="inlineStr">
+        <is>
+          <t>Not sure / not applicable to my role — I don’t have visibility into this</t>
+        </is>
+      </c>
     </row>
     <row r="93">
       <c r="A93" s="2" t="inlineStr">
@@ -14094,6 +15398,11 @@
           <t>All regulatory-relevant logs on certified immutable storage with cryptographic integrity checks.</t>
         </is>
       </c>
+      <c r="K93" s="2" t="inlineStr">
+        <is>
+          <t>Not sure / not applicable to my role — I don’t have visibility into this</t>
+        </is>
+      </c>
     </row>
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
@@ -14146,6 +15455,11 @@
           <t>Within hours — automated audit-pack generation with a full chain of custody.</t>
         </is>
       </c>
+      <c r="K94" s="2" t="inlineStr">
+        <is>
+          <t>Not sure / not applicable to my role — I don’t have visibility into this</t>
+        </is>
+      </c>
     </row>
     <row r="95">
       <c r="A95" s="2" t="inlineStr">
@@ -14198,6 +15512,11 @@
           <t>Zero-trust log access with MFA, just-in-time provisioning, and real-time access alerts.</t>
         </is>
       </c>
+      <c r="K95" s="2" t="inlineStr">
+        <is>
+          <t>Not sure / not applicable to my role — I don’t have visibility into this</t>
+        </is>
+      </c>
     </row>
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
@@ -14250,6 +15569,11 @@
           <t>Zero data egress enforced technically — all logs ingested, processed, and stored within the organisation perimeter.</t>
         </is>
       </c>
+      <c r="K96" s="2" t="inlineStr">
+        <is>
+          <t>Not sure / not applicable to my role — I don’t have visibility into this</t>
+        </is>
+      </c>
     </row>
     <row r="97">
       <c r="A97" s="2" t="inlineStr">
@@ -14302,6 +15626,11 @@
           <t>Automated retention controls, immutable storage, and on-demand CBUAE/SAMA regulatory reporting.</t>
         </is>
       </c>
+      <c r="K97" s="2" t="inlineStr">
+        <is>
+          <t>Not sure / not applicable to my role — I don’t have visibility into this</t>
+        </is>
+      </c>
     </row>
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
@@ -14354,6 +15683,11 @@
           <t>All regulatory-relevant logs on certified immutable storage with cryptographic integrity verification.</t>
         </is>
       </c>
+      <c r="K98" s="2" t="inlineStr">
+        <is>
+          <t>Not sure / not applicable to my role — I don’t have visibility into this</t>
+        </is>
+      </c>
     </row>
     <row r="99">
       <c r="A99" s="2" t="inlineStr">
@@ -14406,6 +15740,11 @@
           <t>Within hours — automated audit-pack generation with full chain of custody.</t>
         </is>
       </c>
+      <c r="K99" s="2" t="inlineStr">
+        <is>
+          <t>Not sure / not applicable to my role — I don’t have visibility into this</t>
+        </is>
+      </c>
     </row>
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
@@ -14458,6 +15797,11 @@
           <t>Zero-trust log access with MFA, just-in-time provisioning, and real-time access alerts for sensitive data.</t>
         </is>
       </c>
+      <c r="K100" s="2" t="inlineStr">
+        <is>
+          <t>Not sure / not applicable to my role — I don’t have visibility into this</t>
+        </is>
+      </c>
     </row>
     <row r="101">
       <c r="A101" s="2" t="inlineStr">
@@ -14510,6 +15854,11 @@
           <t>Zero data egress enforced technically — all logs ingested, processed, and stored within the country perimeter.</t>
         </is>
       </c>
+      <c r="K101" s="2" t="inlineStr">
+        <is>
+          <t>Not sure / not applicable to my role — I don’t have visibility into this</t>
+        </is>
+      </c>
     </row>
     <row r="102">
       <c r="A102" s="2" t="inlineStr">
@@ -14562,6 +15911,11 @@
           <t>Automated retention controls, immutable storage, and on-demand regulatory evidence packaging.</t>
         </is>
       </c>
+      <c r="K102" s="2" t="inlineStr">
+        <is>
+          <t>Not sure / not applicable to my role — I don’t have visibility into this</t>
+        </is>
+      </c>
     </row>
     <row r="103">
       <c r="A103" s="2" t="inlineStr">
@@ -14614,6 +15968,11 @@
           <t>All regulatory-relevant logs on certified immutable storage with cryptographic integrity checks.</t>
         </is>
       </c>
+      <c r="K103" s="2" t="inlineStr">
+        <is>
+          <t>Not sure / not applicable to my role — I don’t have visibility into this</t>
+        </is>
+      </c>
     </row>
     <row r="104">
       <c r="A104" s="2" t="inlineStr">
@@ -14666,6 +16025,11 @@
           <t>Within hours — automated audit-pack generation with a full chain of custody.</t>
         </is>
       </c>
+      <c r="K104" s="2" t="inlineStr">
+        <is>
+          <t>Not sure / not applicable to my role — I don’t have visibility into this</t>
+        </is>
+      </c>
     </row>
     <row r="105">
       <c r="A105" s="2" t="inlineStr">
@@ -14718,6 +16082,11 @@
           <t>Zero-trust log access with MFA, just-in-time provisioning, and real-time access alerts for sensitive data.</t>
         </is>
       </c>
+      <c r="K105" s="2" t="inlineStr">
+        <is>
+          <t>Not sure / not applicable to my role — I don’t have visibility into this</t>
+        </is>
+      </c>
     </row>
     <row r="106">
       <c r="A106" s="2" t="inlineStr">
@@ -14770,6 +16139,11 @@
           <t>Zero data egress enforced technically — all logs ingested, processed, and stored within the licensed jurisdiction.</t>
         </is>
       </c>
+      <c r="K106" s="2" t="inlineStr">
+        <is>
+          <t>Not sure / not applicable to my role — I don’t have visibility into this</t>
+        </is>
+      </c>
     </row>
     <row r="107">
       <c r="A107" s="2" t="inlineStr">
@@ -14822,6 +16196,11 @@
           <t>Automated retention controls, immutable storage, and on-demand regulatory and settlement audit packs.</t>
         </is>
       </c>
+      <c r="K107" s="2" t="inlineStr">
+        <is>
+          <t>Not sure / not applicable to my role — I don’t have visibility into this</t>
+        </is>
+      </c>
     </row>
     <row r="108">
       <c r="A108" s="2" t="inlineStr">
@@ -14874,6 +16253,11 @@
           <t>All payment-relevant logs on certified immutable storage with cryptographic integrity verification.</t>
         </is>
       </c>
+      <c r="K108" s="2" t="inlineStr">
+        <is>
+          <t>Not sure / not applicable to my role — I don’t have visibility into this</t>
+        </is>
+      </c>
     </row>
     <row r="109">
       <c r="A109" s="2" t="inlineStr">
@@ -14926,6 +16310,11 @@
           <t>Within hours — automated dispute and audit-pack generation with chain of custody.</t>
         </is>
       </c>
+      <c r="K109" s="2" t="inlineStr">
+        <is>
+          <t>Not sure / not applicable to my role — I don’t have visibility into this</t>
+        </is>
+      </c>
     </row>
     <row r="110">
       <c r="A110" s="2" t="inlineStr">
@@ -14978,6 +16367,11 @@
           <t>Zero-trust access with MFA, just-in-time provisioning, and real-time access alerts for payment data.</t>
         </is>
       </c>
+      <c r="K110" s="2" t="inlineStr">
+        <is>
+          <t>Not sure / not applicable to my role — I don’t have visibility into this</t>
+        </is>
+      </c>
     </row>
     <row r="111">
       <c r="A111" s="2" t="inlineStr">
@@ -15030,6 +16424,11 @@
           <t>Zero data egress enforced technically with continuous compliance monitoring and annual PCI-DSS certification.</t>
         </is>
       </c>
+      <c r="K111" s="2" t="inlineStr">
+        <is>
+          <t>Not sure / not applicable to my role — I don’t have visibility into this</t>
+        </is>
+      </c>
     </row>
     <row r="112">
       <c r="A112" s="2" t="inlineStr">
@@ -15082,6 +16481,11 @@
           <t>Automated retention controls, immutable storage, and on-demand PCI/scheme audit packs.</t>
         </is>
       </c>
+      <c r="K112" s="2" t="inlineStr">
+        <is>
+          <t>Not sure / not applicable to my role — I don’t have visibility into this</t>
+        </is>
+      </c>
     </row>
     <row r="113">
       <c r="A113" s="2" t="inlineStr">
@@ -15134,6 +16538,11 @@
           <t>All in-scope payment logs on certified immutable storage with cryptographic integrity verification.</t>
         </is>
       </c>
+      <c r="K113" s="2" t="inlineStr">
+        <is>
+          <t>Not sure / not applicable to my role — I don’t have visibility into this</t>
+        </is>
+      </c>
     </row>
     <row r="114">
       <c r="A114" s="2" t="inlineStr">
@@ -15186,6 +16595,11 @@
           <t>Within hours — automated dispute and audit-pack generation with chain of custody.</t>
         </is>
       </c>
+      <c r="K114" s="2" t="inlineStr">
+        <is>
+          <t>Not sure / not applicable to my role — I don’t have visibility into this</t>
+        </is>
+      </c>
     </row>
     <row r="115">
       <c r="A115" s="2" t="inlineStr">
@@ -15238,6 +16652,11 @@
           <t>Zero-trust access with MFA, just-in-time provisioning, and real-time alerts for cardholder data access.</t>
         </is>
       </c>
+      <c r="K115" s="2" t="inlineStr">
+        <is>
+          <t>Not sure / not applicable to my role — I don’t have visibility into this</t>
+        </is>
+      </c>
     </row>
     <row r="116">
       <c r="A116" s="2" t="inlineStr">
@@ -15290,6 +16709,11 @@
           <t>Zero data egress enforced technically with continuous compliance monitoring and annual certification.</t>
         </is>
       </c>
+      <c r="K116" s="2" t="inlineStr">
+        <is>
+          <t>Not sure / not applicable to my role — I don’t have visibility into this</t>
+        </is>
+      </c>
     </row>
     <row r="117">
       <c r="A117" s="2" t="inlineStr">
@@ -15342,6 +16766,11 @@
           <t>Automated retention controls, immutable storage, and on-demand audit pack generation for all statutory requirements.</t>
         </is>
       </c>
+      <c r="K117" s="2" t="inlineStr">
+        <is>
+          <t>Not sure / not applicable to my role — I don’t have visibility into this</t>
+        </is>
+      </c>
     </row>
     <row r="118">
       <c r="A118" s="2" t="inlineStr">
@@ -15394,6 +16823,11 @@
           <t>All in-scope logs on certified immutable storage with cryptographic integrity checks and chain of custody.</t>
         </is>
       </c>
+      <c r="K118" s="2" t="inlineStr">
+        <is>
+          <t>Not sure / not applicable to my role — I don’t have visibility into this</t>
+        </is>
+      </c>
     </row>
     <row r="119">
       <c r="A119" s="2" t="inlineStr">
@@ -15446,6 +16880,11 @@
           <t>Within hours — automated audit pack generation with full chain of custody for statutory submissions.</t>
         </is>
       </c>
+      <c r="K119" s="2" t="inlineStr">
+        <is>
+          <t>Not sure / not applicable to my role — I don’t have visibility into this</t>
+        </is>
+      </c>
     </row>
     <row r="120">
       <c r="A120" s="2" t="inlineStr">
@@ -15498,6 +16937,11 @@
           <t>Zero-trust log access with MFA, just-in-time provisioning, and automated alerts for sensitive data access.</t>
         </is>
       </c>
+      <c r="K120" s="2" t="inlineStr">
+        <is>
+          <t>Not sure / not applicable to my role — I don’t have visibility into this</t>
+        </is>
+      </c>
     </row>
     <row r="121">
       <c r="A121" s="2" t="inlineStr">
@@ -15550,6 +16994,11 @@
           <t>Zero data egress enforced technically — all logs ingested, processed, and stored within approved government infrastructure.</t>
         </is>
       </c>
+      <c r="K121" s="2" t="inlineStr">
+        <is>
+          <t>Not sure / not applicable to my role — I don’t have visibility into this</t>
+        </is>
+      </c>
     </row>
     <row r="122">
       <c r="A122" s="2" t="inlineStr">
@@ -15602,6 +17051,11 @@
           <t>Automated retention controls, immutable storage, and on-demand audit pack generation for all statutory requirements.</t>
         </is>
       </c>
+      <c r="K122" s="2" t="inlineStr">
+        <is>
+          <t>Not sure / not applicable to my role — I don’t have visibility into this</t>
+        </is>
+      </c>
     </row>
     <row r="123">
       <c r="A123" s="2" t="inlineStr">
@@ -15654,6 +17108,11 @@
           <t>All in-scope logs on certified immutable storage with cryptographic integrity checks and chain of custody.</t>
         </is>
       </c>
+      <c r="K123" s="2" t="inlineStr">
+        <is>
+          <t>Not sure / not applicable to my role — I don’t have visibility into this</t>
+        </is>
+      </c>
     </row>
     <row r="124">
       <c r="A124" s="2" t="inlineStr">
@@ -15706,6 +17165,11 @@
           <t>Within hours — automated audit pack generation with full chain of custody for statutory submissions.</t>
         </is>
       </c>
+      <c r="K124" s="2" t="inlineStr">
+        <is>
+          <t>Not sure / not applicable to my role — I don’t have visibility into this</t>
+        </is>
+      </c>
     </row>
     <row r="125">
       <c r="A125" s="2" t="inlineStr">
@@ -15758,6 +17222,11 @@
           <t>Zero-trust log access with MFA, just-in-time provisioning, and automated alerts for sensitive citizen data access.</t>
         </is>
       </c>
+      <c r="K125" s="2" t="inlineStr">
+        <is>
+          <t>Not sure / not applicable to my role — I don’t have visibility into this</t>
+        </is>
+      </c>
     </row>
     <row r="126">
       <c r="A126" s="2" t="inlineStr">
@@ -15810,6 +17279,11 @@
           <t>Zero data egress enforced technically — all logs ingested, processed, and stored within approved sovereign infrastructure.</t>
         </is>
       </c>
+      <c r="K126" s="2" t="inlineStr">
+        <is>
+          <t>Not sure / not applicable to my role — I don’t have visibility into this</t>
+        </is>
+      </c>
     </row>
     <row r="127">
       <c r="A127" s="2" t="inlineStr">
@@ -15862,6 +17336,11 @@
           <t>Automated retention controls, immutable storage, and on-demand audit evidence generation for all certification scopes.</t>
         </is>
       </c>
+      <c r="K127" s="2" t="inlineStr">
+        <is>
+          <t>Not sure / not applicable to my role — I don’t have visibility into this</t>
+        </is>
+      </c>
     </row>
     <row r="128">
       <c r="A128" s="2" t="inlineStr">
@@ -15914,6 +17393,11 @@
           <t>All in-scope logs on certified immutable storage with cryptographic integrity verification.</t>
         </is>
       </c>
+      <c r="K128" s="2" t="inlineStr">
+        <is>
+          <t>Not sure / not applicable to my role — I don’t have visibility into this</t>
+        </is>
+      </c>
     </row>
     <row r="129">
       <c r="A129" s="2" t="inlineStr">
@@ -15966,6 +17450,11 @@
           <t>Within hours — automated evidence package generation with full chain of custody.</t>
         </is>
       </c>
+      <c r="K129" s="2" t="inlineStr">
+        <is>
+          <t>Not sure / not applicable to my role — I don’t have visibility into this</t>
+        </is>
+      </c>
     </row>
     <row r="130">
       <c r="A130" s="2" t="inlineStr">
@@ -16018,6 +17507,11 @@
           <t>Zero-trust log access with MFA, just-in-time provisioning, and automated alerts for sensitive data access.</t>
         </is>
       </c>
+      <c r="K130" s="2" t="inlineStr">
+        <is>
+          <t>Not sure / not applicable to my role — I don’t have visibility into this</t>
+        </is>
+      </c>
     </row>
     <row r="131">
       <c r="A131" s="2" t="inlineStr">
@@ -16070,6 +17564,11 @@
           <t>Zero data egress enforced technically — all logs ingested, processed, and stored within contractually required boundaries.</t>
         </is>
       </c>
+      <c r="K131" s="2" t="inlineStr">
+        <is>
+          <t>Not sure / not applicable to my role — I don’t have visibility into this</t>
+        </is>
+      </c>
     </row>
     <row r="132">
       <c r="A132" s="2" t="inlineStr">
@@ -16122,6 +17621,11 @@
           <t>Automated retention controls, immutable storage, and on-demand PCI-DSS and DPDP audit evidence.</t>
         </is>
       </c>
+      <c r="K132" s="2" t="inlineStr">
+        <is>
+          <t>Not sure / not applicable to my role — I don’t have visibility into this</t>
+        </is>
+      </c>
     </row>
     <row r="133">
       <c r="A133" s="2" t="inlineStr">
@@ -16174,6 +17678,11 @@
           <t>All in-scope logs on certified immutable storage with cryptographic integrity verification.</t>
         </is>
       </c>
+      <c r="K133" s="2" t="inlineStr">
+        <is>
+          <t>Not sure / not applicable to my role — I don’t have visibility into this</t>
+        </is>
+      </c>
     </row>
     <row r="134">
       <c r="A134" s="2" t="inlineStr">
@@ -16226,6 +17735,11 @@
           <t>Within hours — automated evidence package generation with full chain of custody.</t>
         </is>
       </c>
+      <c r="K134" s="2" t="inlineStr">
+        <is>
+          <t>Not sure / not applicable to my role — I don’t have visibility into this</t>
+        </is>
+      </c>
     </row>
     <row r="135">
       <c r="A135" s="2" t="inlineStr">
@@ -16278,6 +17792,11 @@
           <t>Zero-trust log access with MFA, just-in-time provisioning, and automated alerts for customer data access.</t>
         </is>
       </c>
+      <c r="K135" s="2" t="inlineStr">
+        <is>
+          <t>Not sure / not applicable to my role — I don’t have visibility into this</t>
+        </is>
+      </c>
     </row>
     <row r="136">
       <c r="A136" s="2" t="inlineStr">
@@ -16330,6 +17849,11 @@
           <t>Zero data egress enforced technically with continuous compliance monitoring and PCI-DSS certification.</t>
         </is>
       </c>
+      <c r="K136" s="2" t="inlineStr">
+        <is>
+          <t>Not sure / not applicable to my role — I don’t have visibility into this</t>
+        </is>
+      </c>
     </row>
     <row r="137">
       <c r="A137" s="2" t="inlineStr">
@@ -16382,6 +17906,11 @@
           <t>Automated retention controls, immutable storage, and on-demand PCI-DSS and data protection audit evidence.</t>
         </is>
       </c>
+      <c r="K137" s="2" t="inlineStr">
+        <is>
+          <t>Not sure / not applicable to my role — I don’t have visibility into this</t>
+        </is>
+      </c>
     </row>
     <row r="138">
       <c r="A138" s="2" t="inlineStr">
@@ -16434,6 +17963,11 @@
           <t>All in-scope logs on certified immutable storage with cryptographic integrity verification.</t>
         </is>
       </c>
+      <c r="K138" s="2" t="inlineStr">
+        <is>
+          <t>Not sure / not applicable to my role — I don’t have visibility into this</t>
+        </is>
+      </c>
     </row>
     <row r="139">
       <c r="A139" s="2" t="inlineStr">
@@ -16486,6 +18020,11 @@
           <t>Within hours — automated evidence package generation with full chain of custody.</t>
         </is>
       </c>
+      <c r="K139" s="2" t="inlineStr">
+        <is>
+          <t>Not sure / not applicable to my role — I don’t have visibility into this</t>
+        </is>
+      </c>
     </row>
     <row r="140">
       <c r="A140" s="2" t="inlineStr">
@@ -16538,6 +18077,11 @@
           <t>Zero-trust log access with MFA, just-in-time provisioning, and automated alerts for customer data access.</t>
         </is>
       </c>
+      <c r="K140" s="2" t="inlineStr">
+        <is>
+          <t>Not sure / not applicable to my role — I don’t have visibility into this</t>
+        </is>
+      </c>
     </row>
     <row r="141">
       <c r="A141" s="2" t="inlineStr">
@@ -16590,6 +18134,11 @@
           <t>Zero data egress enforced technically with continuous compliance monitoring and PCI-DSS certification.</t>
         </is>
       </c>
+      <c r="K141" s="2" t="inlineStr">
+        <is>
+          <t>Not sure / not applicable to my role — I don’t have visibility into this</t>
+        </is>
+      </c>
     </row>
     <row r="142">
       <c r="A142" s="2" t="inlineStr">
@@ -16642,6 +18191,11 @@
           <t>Automated retention controls, immutable storage, and on-demand DoT/TRAI/CERT-In audit packs.</t>
         </is>
       </c>
+      <c r="K142" s="2" t="inlineStr">
+        <is>
+          <t>Not sure / not applicable to my role — I don’t have visibility into this</t>
+        </is>
+      </c>
     </row>
     <row r="143">
       <c r="A143" s="2" t="inlineStr">
@@ -16694,6 +18248,11 @@
           <t>All DoT-mandated records on certified immutable storage with cryptographic integrity and chain of custody.</t>
         </is>
       </c>
+      <c r="K143" s="2" t="inlineStr">
+        <is>
+          <t>Not sure / not applicable to my role — I don’t have visibility into this</t>
+        </is>
+      </c>
     </row>
     <row r="144">
       <c r="A144" s="2" t="inlineStr">
@@ -16746,6 +18305,11 @@
           <t>Within hours — automated audit-pack and lawful interception evidence generation with full chain of custody.</t>
         </is>
       </c>
+      <c r="K144" s="2" t="inlineStr">
+        <is>
+          <t>Not sure / not applicable to my role — I don’t have visibility into this</t>
+        </is>
+      </c>
     </row>
     <row r="145">
       <c r="A145" s="2" t="inlineStr">
@@ -16798,6 +18362,11 @@
           <t>Zero-trust access with MFA, just-in-time provisioning, and automated alerts for sensitive subscriber data access.</t>
         </is>
       </c>
+      <c r="K145" s="2" t="inlineStr">
+        <is>
+          <t>Not sure / not applicable to my role — I don’t have visibility into this</t>
+        </is>
+      </c>
     </row>
     <row r="146">
       <c r="A146" s="2" t="inlineStr">
@@ -16850,6 +18419,11 @@
           <t>Zero data egress enforced technically — all subscriber data and CDRs ingested, processed, and stored within Indian jurisdiction.</t>
         </is>
       </c>
+      <c r="K146" s="2" t="inlineStr">
+        <is>
+          <t>Not sure / not applicable to my role — I don’t have visibility into this</t>
+        </is>
+      </c>
     </row>
     <row r="147">
       <c r="A147" s="2" t="inlineStr">
@@ -16902,6 +18476,11 @@
           <t>Automated retention controls, immutable storage, and on-demand regulator and law enforcement audit packs.</t>
         </is>
       </c>
+      <c r="K147" s="2" t="inlineStr">
+        <is>
+          <t>Not sure / not applicable to my role — I don’t have visibility into this</t>
+        </is>
+      </c>
     </row>
     <row r="148">
       <c r="A148" s="2" t="inlineStr">
@@ -16954,6 +18533,11 @@
           <t>All legally mandated records on certified immutable storage with cryptographic integrity and chain of custody.</t>
         </is>
       </c>
+      <c r="K148" s="2" t="inlineStr">
+        <is>
+          <t>Not sure / not applicable to my role — I don’t have visibility into this</t>
+        </is>
+      </c>
     </row>
     <row r="149">
       <c r="A149" s="2" t="inlineStr">
@@ -17006,6 +18590,11 @@
           <t>Within hours — automated audit-pack and lawful interception evidence generation with full chain of custody.</t>
         </is>
       </c>
+      <c r="K149" s="2" t="inlineStr">
+        <is>
+          <t>Not sure / not applicable to my role — I don’t have visibility into this</t>
+        </is>
+      </c>
     </row>
     <row r="150">
       <c r="A150" s="2" t="inlineStr">
@@ -17058,6 +18647,11 @@
           <t>Zero-trust access with MFA, just-in-time provisioning, and automated alerts for sensitive subscriber data access.</t>
         </is>
       </c>
+      <c r="K150" s="2" t="inlineStr">
+        <is>
+          <t>Not sure / not applicable to my role — I don’t have visibility into this</t>
+        </is>
+      </c>
     </row>
     <row r="151">
       <c r="A151" s="2" t="inlineStr">
@@ -17110,6 +18704,11 @@
           <t>Zero data egress enforced technically — all subscriber data and CDRs stored within applicable jurisdictional boundaries.</t>
         </is>
       </c>
+      <c r="K151" s="2" t="inlineStr">
+        <is>
+          <t>Not sure / not applicable to my role — I don’t have visibility into this</t>
+        </is>
+      </c>
     </row>
     <row r="152">
       <c r="A152" s="2" t="inlineStr">
@@ -17162,6 +18761,11 @@
           <t>Automated retention controls, immutable storage, and on-demand CERC/SERC/CERT-In audit packs.</t>
         </is>
       </c>
+      <c r="K152" s="2" t="inlineStr">
+        <is>
+          <t>Not sure / not applicable to my role — I don’t have visibility into this</t>
+        </is>
+      </c>
     </row>
     <row r="153">
       <c r="A153" s="2" t="inlineStr">
@@ -17214,6 +18818,11 @@
           <t>All CII-relevant logs on certified immutable storage with cryptographic integrity checks and chain of custody.</t>
         </is>
       </c>
+      <c r="K153" s="2" t="inlineStr">
+        <is>
+          <t>Not sure / not applicable to my role — I don’t have visibility into this</t>
+        </is>
+      </c>
     </row>
     <row r="154">
       <c r="A154" s="2" t="inlineStr">
@@ -17266,6 +18875,11 @@
           <t>Within hours — automated audit pack generation with full chain of custody for regulatory submissions.</t>
         </is>
       </c>
+      <c r="K154" s="2" t="inlineStr">
+        <is>
+          <t>Not sure / not applicable to my role — I don’t have visibility into this</t>
+        </is>
+      </c>
     </row>
     <row r="155">
       <c r="A155" s="2" t="inlineStr">
@@ -17318,6 +18932,11 @@
           <t>Zero-trust access across OT and IT with MFA, just-in-time provisioning, and automated alerts for sensitive access.</t>
         </is>
       </c>
+      <c r="K155" s="2" t="inlineStr">
+        <is>
+          <t>Not sure / not applicable to my role — I don’t have visibility into this</t>
+        </is>
+      </c>
     </row>
     <row r="156">
       <c r="A156" s="2" t="inlineStr">
@@ -17370,6 +18989,11 @@
           <t>Zero data egress enforced technically — all operational and consumer data stored within Indian jurisdiction.</t>
         </is>
       </c>
+      <c r="K156" s="2" t="inlineStr">
+        <is>
+          <t>Not sure / not applicable to my role — I don’t have visibility into this</t>
+        </is>
+      </c>
     </row>
     <row r="157">
       <c r="A157" s="2" t="inlineStr">
@@ -17422,6 +19046,11 @@
           <t>Automated retention controls, immutable storage, and on-demand regulatory audit packs.</t>
         </is>
       </c>
+      <c r="K157" s="2" t="inlineStr">
+        <is>
+          <t>Not sure / not applicable to my role — I don’t have visibility into this</t>
+        </is>
+      </c>
     </row>
     <row r="158">
       <c r="A158" s="2" t="inlineStr">
@@ -17474,6 +19103,11 @@
           <t>All in-scope logs on certified immutable storage with cryptographic integrity checks and chain of custody.</t>
         </is>
       </c>
+      <c r="K158" s="2" t="inlineStr">
+        <is>
+          <t>Not sure / not applicable to my role — I don’t have visibility into this</t>
+        </is>
+      </c>
     </row>
     <row r="159">
       <c r="A159" s="2" t="inlineStr">
@@ -17526,6 +19160,11 @@
           <t>Within hours — automated audit pack generation with full chain of custody for regulatory submissions.</t>
         </is>
       </c>
+      <c r="K159" s="2" t="inlineStr">
+        <is>
+          <t>Not sure / not applicable to my role — I don’t have visibility into this</t>
+        </is>
+      </c>
     </row>
     <row r="160">
       <c r="A160" s="2" t="inlineStr">
@@ -17578,6 +19217,11 @@
           <t>Zero-trust access across OT and IT with MFA, just-in-time provisioning, and automated alerts for sensitive access.</t>
         </is>
       </c>
+      <c r="K160" s="2" t="inlineStr">
+        <is>
+          <t>Not sure / not applicable to my role — I don’t have visibility into this</t>
+        </is>
+      </c>
     </row>
     <row r="161">
       <c r="A161" s="2" t="inlineStr">
@@ -17630,6 +19274,11 @@
           <t>Zero data egress enforced technically — all operational and consumer data stored within applicable jurisdictional boundaries.</t>
         </is>
       </c>
+      <c r="K161" s="2" t="inlineStr">
+        <is>
+          <t>Not sure / not applicable to my role — I don’t have visibility into this</t>
+        </is>
+      </c>
     </row>
     <row r="162">
       <c r="A162" s="2" t="inlineStr">
@@ -17682,6 +19331,11 @@
           <t>Automated retention controls, immutable storage, and on-demand evidence generation for all certification and regulatory scopes.</t>
         </is>
       </c>
+      <c r="K162" s="2" t="inlineStr">
+        <is>
+          <t>Not sure / not applicable to my role — I don’t have visibility into this</t>
+        </is>
+      </c>
     </row>
     <row r="163">
       <c r="A163" s="2" t="inlineStr">
@@ -17734,6 +19388,11 @@
           <t>All regulated production records on certified immutable storage with cryptographic integrity verification.</t>
         </is>
       </c>
+      <c r="K163" s="2" t="inlineStr">
+        <is>
+          <t>Not sure / not applicable to my role — I don’t have visibility into this</t>
+        </is>
+      </c>
     </row>
     <row r="164">
       <c r="A164" s="2" t="inlineStr">
@@ -17786,6 +19445,11 @@
           <t>Within hours — automated evidence package generation with full production batch chain of custody.</t>
         </is>
       </c>
+      <c r="K164" s="2" t="inlineStr">
+        <is>
+          <t>Not sure / not applicable to my role — I don’t have visibility into this</t>
+        </is>
+      </c>
     </row>
     <row r="165">
       <c r="A165" s="2" t="inlineStr">
@@ -17838,6 +19502,11 @@
           <t>Zero-trust access with MFA, just-in-time provisioning, and automated alerts for sensitive production data access.</t>
         </is>
       </c>
+      <c r="K165" s="2" t="inlineStr">
+        <is>
+          <t>Not sure / not applicable to my role — I don’t have visibility into this</t>
+        </is>
+      </c>
     </row>
     <row r="166">
       <c r="A166" s="2" t="inlineStr">
@@ -17888,6 +19557,11 @@
       <c r="J166" s="2" t="inlineStr">
         <is>
           <t>Full data lifecycle governance — production records, quality data, and supply chain data retained, protected, and accessible for audit, recall, and ESG reporting.</t>
+        </is>
+      </c>
+      <c r="K166" s="2" t="inlineStr">
+        <is>
+          <t>Not sure / not applicable to my role — I don’t have visibility into this</t>
         </is>
       </c>
     </row>

</xml_diff>